<commit_message>
Figura de PEP por registro contra UCS referencial, ROP y PP; hoja de Spearman de la PEP en el Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT9AkNnHr1e9AMWji6YncB
</commit_message>
<xml_diff>
--- a/figuras/finales/tablas_capitulo6.xlsx
+++ b/figuras/finales/tablas_capitulo6.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="256">
   <si>
     <t xml:space="preserve">Configuración de la corrida final (2026-10-22)</t>
   </si>
@@ -531,6 +531,21 @@
     <t xml:space="preserve">220–230</t>
   </si>
   <si>
+    <t xml:space="preserve">Correlación de Spearman de la PEP por registro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ρ de Spearman con la PEP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS referencial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">717.526 registros entrenables de roca intacta con PEP ≤ 1000 y ROP ≥ 0.2 m/min; 506 excluidos por PEP &gt; 1000 (ROP ≈ 0).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Picos de DI y cruces de malla en PCC_1541 (radio 3 m)</t>
   </si>
   <si>
@@ -738,7 +753,7 @@
     <t xml:space="preserve">PCC_0042_PR01_TH_P49_H6</t>
   </si>
   <si>
-    <t xml:space="preserve">Modelo de bloques de 2.5 m (IDW)</t>
+    <t xml:space="preserve">Modelo de bloques de 2,5 m (IDW)</t>
   </si>
   <si>
     <t xml:space="preserve">Bloques</t>
@@ -1702,11 +1717,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
@@ -3004,6 +3018,48 @@
       </c>
       <c r="G57" s="23" t="n">
         <v>1.109</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B61" s="17" t="n">
+        <v>0.203</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B62" s="19" t="n">
+        <v>-0.904</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B63" s="17" t="n">
+        <v>0.071</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="12" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -3036,30 +3092,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3256,20 +3312,20 @@
     </row>
     <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>1320</v>
@@ -3285,7 +3341,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B16" s="34" t="n">
         <v>0.152</v>
@@ -3328,41 +3384,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>164.932209858122</v>
@@ -3379,13 +3435,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D4" s="15" t="n">
         <v>138.496561143358</v>
@@ -3402,13 +3458,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>134.789098647061</v>
@@ -3425,13 +3481,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>191</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>186</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>154.123768904038</v>
@@ -3448,13 +3504,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>137.155726282</v>
@@ -3471,13 +3527,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>188</v>
-      </c>
       <c r="C8" s="4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>139.393544557154</v>
@@ -3494,13 +3550,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>153.727676276695</v>
@@ -3517,13 +3573,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>168.41475157952</v>
@@ -3540,13 +3596,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>144.172700603197</v>
@@ -3563,13 +3619,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>159.684160752595</v>
@@ -3586,13 +3642,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>167.800529418651</v>
@@ -3609,13 +3665,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>124.601455398543</v>
@@ -3632,13 +3688,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>119.768508894793</v>
@@ -3655,13 +3711,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>119.704137883813</v>
@@ -3678,13 +3734,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>158.678228976082</v>
@@ -3701,7 +3757,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -3735,45 +3791,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>149</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>34</v>
@@ -3781,7 +3837,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B3" s="16" t="n">
         <v>1</v>
@@ -3811,7 +3867,7 @@
         <v>0.0048</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="L3" s="14" t="n">
         <v>18.033</v>
@@ -3822,7 +3878,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>2</v>
@@ -3852,7 +3908,7 @@
         <v>0.0095</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="L4" s="15" t="n">
         <v>23.376</v>
@@ -3863,7 +3919,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>3</v>
@@ -3893,7 +3949,7 @@
         <v>0.0117</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="L5" s="14" t="n">
         <v>10.993</v>
@@ -3904,7 +3960,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>4</v>
@@ -3934,7 +3990,7 @@
         <v>0.0128</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="L6" s="15" t="n">
         <v>28.854</v>
@@ -3945,7 +4001,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>5</v>
@@ -3975,7 +4031,7 @@
         <v>0.0172</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="L7" s="14" t="n">
         <v>17.351</v>
@@ -3986,7 +4042,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>1</v>
@@ -4016,7 +4072,7 @@
         <v>0.1651</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="L8" s="15" t="n">
         <v>20.324</v>
@@ -4027,7 +4083,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>2</v>
@@ -4057,7 +4113,7 @@
         <v>0.2719</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="L9" s="14" t="n">
         <v>26.594</v>
@@ -4068,7 +4124,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>3</v>
@@ -4098,7 +4154,7 @@
         <v>0.0715</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>19.494</v>
@@ -4109,7 +4165,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>4</v>
@@ -4139,7 +4195,7 @@
         <v>0.0977</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="L11" s="14" t="n">
         <v>18.798</v>
@@ -4150,7 +4206,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>5</v>
@@ -4180,7 +4236,7 @@
         <v>0.1226</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="L12" s="15" t="n">
         <v>20.774</v>
@@ -4191,7 +4247,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>1</v>
@@ -4221,7 +4277,7 @@
         <v>0.1226</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="L13" s="14" t="n">
         <v>20.774</v>
@@ -4232,7 +4288,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B14" s="18" t="n">
         <v>2</v>
@@ -4262,7 +4318,7 @@
         <v>0.1651</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="L14" s="15" t="n">
         <v>20.324</v>
@@ -4273,7 +4329,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>3</v>
@@ -4303,7 +4359,7 @@
         <v>0.1055</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="L15" s="14" t="n">
         <v>28.608</v>
@@ -4314,7 +4370,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>4</v>
@@ -4344,7 +4400,7 @@
         <v>0.0952</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="L16" s="15" t="n">
         <v>20.049</v>
@@ -4355,7 +4411,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>5</v>
@@ -4385,7 +4441,7 @@
         <v>0.0423</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="L17" s="14" t="n">
         <v>28.47</v>
@@ -4421,7 +4477,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4429,13 +4485,13 @@
         <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4509,7 +4565,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>2</v>
@@ -4517,7 +4573,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>233015.6</v>
@@ -4525,7 +4581,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B11" s="29" t="n">
         <v>0.085</v>
@@ -4533,7 +4589,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>0.73</v>
@@ -4541,7 +4597,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B13" s="36" t="n">
         <v>154.4</v>
@@ -4549,7 +4605,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B14" s="35" t="n">
         <v>130.9</v>
@@ -4557,7 +4613,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B15" s="36" t="n">
         <v>170.2</v>
@@ -4565,26 +4621,26 @@
     </row>
     <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C19" s="7" t="n">
         <v>1159</v>
@@ -4592,10 +4648,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>13651</v>
@@ -4603,10 +4659,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>103</v>
@@ -4614,7 +4670,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Comparacion de los cuatro metodos de UCS bajo LOOCV-Caseron: figura, hoja Excel y cifras
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT9AkNnHr1e9AMWji6YncB
</commit_message>
<xml_diff>
--- a/figuras/finales/tablas_capitulo6.xlsx
+++ b/figuras/finales/tablas_capitulo6.xlsx
@@ -15,14 +15,15 @@
     <sheet name="T6.2 Radio RQD" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="GroupKFold" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="LOOCV-Caserón" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Importancia" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Comparación" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="UCS por litología" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="PEP estratos" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="Concordancia 1541" sheetId="12" state="visible" r:id="rId14"/>
-    <sheet name="T6.3 Dominios" sheetId="13" state="visible" r:id="rId15"/>
-    <sheet name="T6.4 Ranking" sheetId="14" state="visible" r:id="rId16"/>
-    <sheet name="Bloques" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="LOOCV-Caserón métodos" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Importancia" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Comparación" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="UCS por litología" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="PEP estratos" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Concordancia 1541" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="T6.3 Dominios" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="T6.4 Ranking" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="Bloques" sheetId="16" state="visible" r:id="rId18"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="285">
   <si>
     <t xml:space="preserve">Configuración de la corrida final (2026-10-22)</t>
   </si>
@@ -364,6 +365,93 @@
   </si>
   <si>
     <t xml:space="preserve">PCS_1059 tiene una sola etiqueta en la prueba: R² y ρ de Spearman indefinidos (celda vacía); AVERAGE los omite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparación de métodos de UCS · LOOCV-Caserón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Método</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etiquetas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAE [MPa]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r de Pearson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Línea base (media litología)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banda por unidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relación directa PEP↔UCS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ML (Random Forest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media de los caserones (correlaciones: solo los definidos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celdas vacías: correlación indefinida (PCS_1059 tiene una sola etiqueta; la línea base predice un valor constante).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relación directa: da un valor por litología; en un caserón con dos litologías su correlación es ±1 por construcción (PCC_0042 +1, PCC_1541 −1): solo dice si ordenó bien las dos, no cuánto acierta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banda y relación: curva PEP→UCS ajustada sin el caserón, evaluada en la PEP mediana de cada litología del caserón excluido; la banda aparta cada registro del centro según su PEP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Curva PEP→UCS de cada pliegue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coeficientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pares (PEP mediana, UCS referencial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extrapola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lineal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3075, 6.872</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(330.9, 128.1); (453.3, 111.5); (386.7, 180.0); (299.3, 60.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.343, 272.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(344.1, 128.1); (453.3, 111.5); (363.1, 180.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bht, Kpcls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.948, -514</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(322.1, 128.1); (359.1, 180.0); (299.3, 60.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brecha_mixta, Kpcli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1984, 48.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(332.4, 128.1); (453.3, 111.5); (359.7, 180.0); (299.3, 60.0)</t>
   </si>
   <si>
     <t xml:space="preserve">Importancia por permutación de las predictoras</t>
@@ -1519,186 +1607,169 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>153</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>34</v>
+        <v>149</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>66</v>
+        <v>154</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B3" s="7" t="n">
-        <v>52992</v>
-      </c>
-      <c r="C3" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="D3" s="14" t="n">
-        <v>115.7</v>
+        <v>159</v>
+      </c>
+      <c r="B3" s="23" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="C3" s="17" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="D3" s="23" t="n">
+        <v>0.04</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>133</v>
+        <v>33.5</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>155.7</v>
-      </c>
-      <c r="G3" s="25" t="n">
-        <f aca="false">E3-C3</f>
-        <v>73</v>
+        <v>5</v>
+      </c>
+      <c r="G3" s="23" t="n">
+        <f aca="false">B3-C3</f>
+        <v>0.048</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="10" t="n">
-        <v>16787</v>
-      </c>
-      <c r="C4" s="15" t="n">
-        <v>111.5</v>
-      </c>
-      <c r="D4" s="15" t="n">
-        <v>145</v>
+        <v>160</v>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>0.703</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="D4" s="24" t="n">
+        <v>0.222</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>154.6</v>
+        <v>36.5</v>
       </c>
       <c r="F4" s="15" t="n">
-        <v>160.4</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <f aca="false">E4-C4</f>
-        <v>43.1</v>
+        <v>3.7</v>
+      </c>
+      <c r="G4" s="24" t="n">
+        <f aca="false">B4-C4</f>
+        <v>0.762</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>224091</v>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>128.1</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>126.7</v>
+        <v>20</v>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>0.485</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>0.189</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>137.6</v>
+        <v>32.4</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>164.3</v>
-      </c>
-      <c r="G5" s="25" t="n">
-        <f aca="false">E5-C5</f>
-        <v>9.5</v>
+        <v>3.6</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <f aca="false">B5-C5</f>
+        <v>0.319</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>424168</v>
-      </c>
-      <c r="C6" s="15" t="n">
-        <v>180</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>140.1</v>
+        <v>161</v>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>0.594</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>0.227</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>167.3</v>
+        <v>32.6</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>177.3</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <f aca="false">E6-C6</f>
-        <v>-12.7</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>140</v>
+        <v>4.1</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <f aca="false">B6-C6</f>
+        <v>0.447</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>0.492</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>0.088</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <f aca="false">B7-C7</f>
+        <v>0.404</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>735674</v>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>32.27</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>29.8</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="B11" s="10" t="n">
-        <v>150985</v>
-      </c>
-      <c r="C11" s="15" t="n">
-        <v>38.32</v>
-      </c>
-      <c r="D11" s="15" t="n">
-        <v>35.7</v>
+      <c r="A9" s="12" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -1717,6 +1788,204 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>52992</v>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>115.7</v>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>133</v>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>155.7</v>
+      </c>
+      <c r="G3" s="25" t="n">
+        <f aca="false">E3-C3</f>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>16787</v>
+      </c>
+      <c r="C4" s="15" t="n">
+        <v>111.5</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>145</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>154.6</v>
+      </c>
+      <c r="F4" s="15" t="n">
+        <v>160.4</v>
+      </c>
+      <c r="G4" s="26" t="n">
+        <f aca="false">E4-C4</f>
+        <v>43.1</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>224091</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>128.1</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>126.7</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>137.6</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>164.3</v>
+      </c>
+      <c r="G5" s="25" t="n">
+        <f aca="false">E5-C5</f>
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>424168</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>180</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>140.1</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>167.3</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>177.3</v>
+      </c>
+      <c r="G6" s="26" t="n">
+        <f aca="false">E6-C6</f>
+        <v>-12.7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>735674</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>32.27</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>150985</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>38.32</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G65"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1729,7 +1998,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1740,19 +2009,19 @@
         <v>66</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>147</v>
+        <v>176</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1763,7 +2032,7 @@
         <v>128.1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>153</v>
@@ -1786,7 +2055,7 @@
         <v>128.1</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>331</v>
@@ -1809,7 +2078,7 @@
         <v>128.1</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>1439</v>
@@ -1832,7 +2101,7 @@
         <v>128.1</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>3303</v>
@@ -1855,7 +2124,7 @@
         <v>128.1</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>6204</v>
@@ -1878,7 +2147,7 @@
         <v>128.1</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>4488</v>
@@ -1901,7 +2170,7 @@
         <v>128.1</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>8306</v>
@@ -1924,7 +2193,7 @@
         <v>128.1</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="D10" s="10" t="n">
         <v>7523</v>
@@ -1947,7 +2216,7 @@
         <v>128.1</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>17670</v>
@@ -1970,7 +2239,7 @@
         <v>128.1</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="D12" s="10" t="n">
         <v>17807</v>
@@ -1993,7 +2262,7 @@
         <v>128.1</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>8826</v>
@@ -2016,7 +2285,7 @@
         <v>128.1</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>17252</v>
@@ -2039,7 +2308,7 @@
         <v>128.1</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>59398</v>
@@ -2062,7 +2331,7 @@
         <v>128.1</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>164</v>
+        <v>193</v>
       </c>
       <c r="D16" s="10" t="n">
         <v>71391</v>
@@ -2085,7 +2354,7 @@
         <v>111.5</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>40</v>
@@ -2108,7 +2377,7 @@
         <v>111.5</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="D18" s="10" t="n">
         <v>54</v>
@@ -2131,7 +2400,7 @@
         <v>111.5</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>106</v>
@@ -2154,7 +2423,7 @@
         <v>111.5</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="D20" s="10" t="n">
         <v>76</v>
@@ -2177,7 +2446,7 @@
         <v>111.5</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>116</v>
@@ -2200,7 +2469,7 @@
         <v>111.5</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="D22" s="10" t="n">
         <v>292</v>
@@ -2223,7 +2492,7 @@
         <v>111.5</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
       <c r="D23" s="7" t="n">
         <v>3030</v>
@@ -2246,7 +2515,7 @@
         <v>111.5</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="D24" s="10" t="n">
         <v>2672</v>
@@ -2269,7 +2538,7 @@
         <v>111.5</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>2282</v>
@@ -2292,7 +2561,7 @@
         <v>111.5</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="D26" s="10" t="n">
         <v>1979</v>
@@ -2315,7 +2584,7 @@
         <v>111.5</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>1986</v>
@@ -2338,7 +2607,7 @@
         <v>111.5</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="D28" s="10" t="n">
         <v>3550</v>
@@ -2361,7 +2630,7 @@
         <v>111.5</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>603</v>
@@ -2384,7 +2653,7 @@
         <v>180</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="D30" s="10" t="n">
         <v>126</v>
@@ -2407,7 +2676,7 @@
         <v>180</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>282</v>
@@ -2430,7 +2699,7 @@
         <v>180</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
       <c r="D32" s="10" t="n">
         <v>738</v>
@@ -2453,7 +2722,7 @@
         <v>180</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="D33" s="7" t="n">
         <v>1542</v>
@@ -2476,7 +2745,7 @@
         <v>180</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D34" s="10" t="n">
         <v>7341</v>
@@ -2499,7 +2768,7 @@
         <v>180</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>7554</v>
@@ -2522,7 +2791,7 @@
         <v>180</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>11164</v>
@@ -2545,7 +2814,7 @@
         <v>180</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="D37" s="7" t="n">
         <v>11833</v>
@@ -2568,7 +2837,7 @@
         <v>180</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
       <c r="D38" s="10" t="n">
         <v>30363</v>
@@ -2591,7 +2860,7 @@
         <v>180</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>16372</v>
@@ -2614,7 +2883,7 @@
         <v>180</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="D40" s="10" t="n">
         <v>10824</v>
@@ -2637,7 +2906,7 @@
         <v>180</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>48445</v>
@@ -2660,7 +2929,7 @@
         <v>180</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="D42" s="10" t="n">
         <v>66162</v>
@@ -2683,7 +2952,7 @@
         <v>180</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>164</v>
+        <v>193</v>
       </c>
       <c r="D43" s="7" t="n">
         <v>211422</v>
@@ -2706,7 +2975,7 @@
         <v>60</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="D44" s="10" t="n">
         <v>34</v>
@@ -2729,7 +2998,7 @@
         <v>60</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="D45" s="7" t="n">
         <v>54</v>
@@ -2752,7 +3021,7 @@
         <v>60</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
       <c r="D46" s="10" t="n">
         <v>410</v>
@@ -2775,7 +3044,7 @@
         <v>60</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="D47" s="7" t="n">
         <v>729</v>
@@ -2798,7 +3067,7 @@
         <v>60</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D48" s="10" t="n">
         <v>971</v>
@@ -2821,7 +3090,7 @@
         <v>60</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="D49" s="7" t="n">
         <v>980</v>
@@ -2844,7 +3113,7 @@
         <v>60</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
       <c r="D50" s="10" t="n">
         <v>736</v>
@@ -2867,7 +3136,7 @@
         <v>60</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="D51" s="7" t="n">
         <v>789</v>
@@ -2890,7 +3159,7 @@
         <v>60</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
       <c r="D52" s="10" t="n">
         <v>4921</v>
@@ -2913,7 +3182,7 @@
         <v>60</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="D53" s="7" t="n">
         <v>3689</v>
@@ -2936,7 +3205,7 @@
         <v>60</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="D54" s="10" t="n">
         <v>1230</v>
@@ -2959,7 +3228,7 @@
         <v>60</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="D55" s="7" t="n">
         <v>6302</v>
@@ -2982,7 +3251,7 @@
         <v>60</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="D56" s="10" t="n">
         <v>7892</v>
@@ -3005,7 +3274,7 @@
         <v>60</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>164</v>
+        <v>193</v>
       </c>
       <c r="D57" s="7" t="n">
         <v>24255</v>
@@ -3022,20 +3291,20 @@
     </row>
     <row r="59" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>165</v>
+        <v>194</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>166</v>
+        <v>195</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>167</v>
+        <v>196</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="B61" s="17" t="n">
         <v>0.203</v>
@@ -3043,7 +3312,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>114</v>
+        <v>143</v>
       </c>
       <c r="B62" s="19" t="n">
         <v>-0.904</v>
@@ -3059,7 +3328,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -3073,7 +3342,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3092,30 +3361,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>172</v>
+        <v>201</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>174</v>
+        <v>203</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>175</v>
+        <v>204</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>177</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3312,20 +3581,20 @@
     </row>
     <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>178</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>179</v>
+        <v>208</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>172</v>
+        <v>201</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>1320</v>
@@ -3341,7 +3610,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="B16" s="34" t="n">
         <v>0.152</v>
@@ -3366,7 +3635,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3384,41 +3653,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>184</v>
+        <v>213</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>185</v>
+        <v>214</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>186</v>
+        <v>215</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>187</v>
+        <v>216</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>189</v>
+        <v>218</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>190</v>
+        <v>219</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>164.932209858122</v>
@@ -3435,13 +3704,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>192</v>
+        <v>221</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D4" s="15" t="n">
         <v>138.496561143358</v>
@@ -3458,13 +3727,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>194</v>
+        <v>223</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>134.789098647061</v>
@@ -3481,13 +3750,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>190</v>
+        <v>219</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>154.123768904038</v>
@@ -3504,13 +3773,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>197</v>
+        <v>226</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>190</v>
+        <v>219</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>137.155726282</v>
@@ -3527,13 +3796,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>139.393544557154</v>
@@ -3550,13 +3819,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>153.727676276695</v>
@@ -3573,13 +3842,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>202</v>
+        <v>231</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>168.41475157952</v>
@@ -3596,13 +3865,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>144.172700603197</v>
@@ -3619,13 +3888,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>204</v>
+        <v>233</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>205</v>
+        <v>234</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>159.684160752595</v>
@@ -3642,13 +3911,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>206</v>
+        <v>235</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>190</v>
+        <v>219</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>205</v>
+        <v>234</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>167.800529418651</v>
@@ -3665,13 +3934,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>207</v>
+        <v>236</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>124.601455398543</v>
@@ -3688,13 +3957,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>119.768508894793</v>
@@ -3711,13 +3980,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>209</v>
+        <v>238</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>119.704137883813</v>
@@ -3734,13 +4003,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>158.678228976082</v>
@@ -3757,7 +4026,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>211</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -3771,7 +4040,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3791,45 +4060,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>213</v>
+        <v>242</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>214</v>
+        <v>243</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>215</v>
+        <v>244</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>216</v>
+        <v>245</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>217</v>
+        <v>246</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>218</v>
+        <v>247</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>220</v>
+        <v>249</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>221</v>
+        <v>250</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>222</v>
+        <v>251</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>223</v>
+        <v>252</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>34</v>
@@ -3837,7 +4106,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="B3" s="16" t="n">
         <v>1</v>
@@ -3867,7 +4136,7 @@
         <v>0.0048</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="L3" s="14" t="n">
         <v>18.033</v>
@@ -3878,7 +4147,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>2</v>
@@ -3908,7 +4177,7 @@
         <v>0.0095</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>226</v>
+        <v>255</v>
       </c>
       <c r="L4" s="15" t="n">
         <v>23.376</v>
@@ -3919,7 +4188,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>3</v>
@@ -3949,7 +4218,7 @@
         <v>0.0117</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>227</v>
+        <v>256</v>
       </c>
       <c r="L5" s="14" t="n">
         <v>10.993</v>
@@ -3960,7 +4229,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>4</v>
@@ -3990,7 +4259,7 @@
         <v>0.0128</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="L6" s="15" t="n">
         <v>28.854</v>
@@ -4001,7 +4270,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>5</v>
@@ -4031,7 +4300,7 @@
         <v>0.0172</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>229</v>
+        <v>258</v>
       </c>
       <c r="L7" s="14" t="n">
         <v>17.351</v>
@@ -4042,7 +4311,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>1</v>
@@ -4072,7 +4341,7 @@
         <v>0.1651</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>231</v>
+        <v>260</v>
       </c>
       <c r="L8" s="15" t="n">
         <v>20.324</v>
@@ -4083,7 +4352,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>2</v>
@@ -4113,7 +4382,7 @@
         <v>0.2719</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>232</v>
+        <v>261</v>
       </c>
       <c r="L9" s="14" t="n">
         <v>26.594</v>
@@ -4124,7 +4393,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>3</v>
@@ -4154,7 +4423,7 @@
         <v>0.0715</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>233</v>
+        <v>262</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>19.494</v>
@@ -4165,7 +4434,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>4</v>
@@ -4195,7 +4464,7 @@
         <v>0.0977</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>233</v>
+        <v>262</v>
       </c>
       <c r="L11" s="14" t="n">
         <v>18.798</v>
@@ -4206,7 +4475,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>5</v>
@@ -4236,7 +4505,7 @@
         <v>0.1226</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>234</v>
+        <v>263</v>
       </c>
       <c r="L12" s="15" t="n">
         <v>20.774</v>
@@ -4247,7 +4516,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>1</v>
@@ -4277,7 +4546,7 @@
         <v>0.1226</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>234</v>
+        <v>263</v>
       </c>
       <c r="L13" s="14" t="n">
         <v>20.774</v>
@@ -4288,7 +4557,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="B14" s="18" t="n">
         <v>2</v>
@@ -4318,7 +4587,7 @@
         <v>0.1651</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>231</v>
+        <v>260</v>
       </c>
       <c r="L14" s="15" t="n">
         <v>20.324</v>
@@ -4329,7 +4598,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>3</v>
@@ -4359,7 +4628,7 @@
         <v>0.1055</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="L15" s="14" t="n">
         <v>28.608</v>
@@ -4370,7 +4639,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>4</v>
@@ -4400,7 +4669,7 @@
         <v>0.0952</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="L16" s="15" t="n">
         <v>20.049</v>
@@ -4411,7 +4680,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>5</v>
@@ -4441,7 +4710,7 @@
         <v>0.0423</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>238</v>
+        <v>267</v>
       </c>
       <c r="L17" s="14" t="n">
         <v>28.47</v>
@@ -4461,7 +4730,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4477,7 +4746,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>239</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4485,13 +4754,13 @@
         <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>241</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4565,7 +4834,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>179</v>
+        <v>208</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>2</v>
@@ -4573,7 +4842,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>233015.6</v>
@@ -4581,7 +4850,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="B11" s="29" t="n">
         <v>0.085</v>
@@ -4589,7 +4858,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>0.73</v>
@@ -4597,7 +4866,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
       <c r="B13" s="36" t="n">
         <v>154.4</v>
@@ -4605,7 +4874,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>246</v>
+        <v>275</v>
       </c>
       <c r="B14" s="35" t="n">
         <v>130.9</v>
@@ -4613,7 +4882,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="B15" s="36" t="n">
         <v>170.2</v>
@@ -4621,26 +4890,26 @@
     </row>
     <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>248</v>
+        <v>277</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>250</v>
+        <v>279</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>251</v>
+        <v>280</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>252</v>
+        <v>281</v>
       </c>
       <c r="C19" s="7" t="n">
         <v>1159</v>
@@ -4648,10 +4917,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>253</v>
+        <v>282</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>252</v>
+        <v>281</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>13651</v>
@@ -4659,10 +4928,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>252</v>
+        <v>281</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>103</v>
@@ -4670,7 +4939,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>255</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -6134,11 +6403,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6151,121 +6426,618 @@
         <v>111</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>112</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="23" t="n">
-        <v>0.2225</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>365416</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>53.64</v>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>49.34</v>
+      </c>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="24" t="n">
-        <v>0.1306</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>131053</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>51.87</v>
+      </c>
+      <c r="F4" s="15" t="n">
+        <v>39.62</v>
+      </c>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B5" s="23" t="n">
-        <v>0.0494</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>122026</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>19.87</v>
+      </c>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>0.0427</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>105108</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B7" s="23" t="n">
-        <v>0.0409</v>
+        <v>116</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>365416</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>73.13</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>64.33</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>0.054</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="B8" s="24" t="n">
-        <v>0.0156</v>
+        <v>116</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>131053</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>88.4</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>0.009</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>-0.04</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="23" t="n">
-        <v>0.0094</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>122026</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>145.25</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>119.6</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>0.057</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>105108</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>62.64</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>56.95</v>
+      </c>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>365416</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>57.71</v>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>54.61</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>131053</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>76.15</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>67.48</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>122026</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>126.86</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>102.28</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>0.066</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>105108</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>365416</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>44.86</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>40.31</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>0.237</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>131053</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>75.86</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>67.26</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H16" s="19" t="n">
+        <v>0.047</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>122026</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>31.59</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>25.51</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>0.048</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>105108</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>49.96</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>48.19</v>
+      </c>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+    </row>
+    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="B22" s="14" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A22,E$3:E$18)</f>
+        <v>48.9</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A22,F$3:F$18)</f>
+        <v>42.2325</v>
+      </c>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="B23" s="15" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A23,E$3:E$18)</f>
+        <v>96.5175</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A23,F$3:F$18)</f>
+        <v>82.32</v>
+      </c>
+      <c r="D23" s="19" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A23,G$3:G$18)</f>
+        <v>0.11</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A23,H$3:H$18)</f>
+        <v>0.0236666666666667</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="B24" s="14" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A24,E$3:E$18)</f>
+        <v>79.53</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A24,F$3:F$18)</f>
+        <v>70.4425</v>
+      </c>
+      <c r="D24" s="17" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A24,G$3:G$18)</f>
+        <v>0.14</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A24,H$3:H$18)</f>
+        <v>0.022</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="23" t="n">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="B15" s="24" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="B25" s="15" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A25,E$3:E$18)</f>
+        <v>50.5675</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A25,F$3:F$18)</f>
+        <v>45.3175</v>
+      </c>
+      <c r="D25" s="19" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A25,G$3:G$18)</f>
+        <v>0.153</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <f aca="false">AVERAGEIF($A$3:$A$18,$A25,H$3:H$18)</f>
+        <v>0.110666666666667</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="B16" s="23" t="n">
-        <v>0.323</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="B17" s="24" t="n">
-        <v>29.7</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="B18" s="23" t="n">
-        <v>723601</v>
+    </row>
+    <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -6284,169 +7056,138 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>130</v>
+        <v>76</v>
       </c>
       <c r="B3" s="23" t="n">
-        <v>0.184</v>
-      </c>
-      <c r="C3" s="17" t="n">
-        <v>0.136</v>
-      </c>
-      <c r="D3" s="23" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="E3" s="14" t="n">
-        <v>33.5</v>
-      </c>
-      <c r="F3" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" s="23" t="n">
-        <f aca="false">B3-C3</f>
-        <v>0.048</v>
+        <v>0.2225</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>131</v>
+        <v>74</v>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.703</v>
-      </c>
-      <c r="C4" s="19" t="n">
-        <v>-0.059</v>
-      </c>
-      <c r="D4" s="24" t="n">
-        <v>0.222</v>
-      </c>
-      <c r="E4" s="15" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="F4" s="15" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="G4" s="24" t="n">
-        <f aca="false">B4-C4</f>
-        <v>0.762</v>
+        <v>0.1306</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B5" s="23" t="n">
-        <v>0.485</v>
-      </c>
-      <c r="C5" s="17" t="n">
-        <v>0.166</v>
-      </c>
-      <c r="D5" s="23" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G5" s="23" t="n">
-        <f aca="false">B5-C5</f>
-        <v>0.319</v>
+        <v>0.0494</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>132</v>
+        <v>73</v>
       </c>
       <c r="B6" s="24" t="n">
-        <v>0.594</v>
-      </c>
-      <c r="C6" s="19" t="n">
-        <v>0.147</v>
-      </c>
-      <c r="D6" s="24" t="n">
-        <v>0.227</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="F6" s="15" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <f aca="false">B6-C6</f>
-        <v>0.447</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>133</v>
+        <v>77</v>
       </c>
       <c r="B7" s="23" t="n">
-        <v>0.492</v>
-      </c>
-      <c r="C7" s="17" t="n">
-        <v>0.088</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>0.214</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G7" s="23" t="n">
-        <f aca="false">B7-C7</f>
-        <v>0.404</v>
+        <v>0.0409</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>0.0156</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>134</v>
+      <c r="A9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>0.0094</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>0.323</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B17" s="24" t="n">
+        <v>29.7</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>723601</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sensibilidad del DI a la ventana: resultados, figura, tabla y hoja Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT9AkNnHr1e9AMWji6YncB
</commit_message>
<xml_diff>
--- a/figuras/finales/tablas_capitulo6.xlsx
+++ b/figuras/finales/tablas_capitulo6.xlsx
@@ -13,17 +13,18 @@
     <sheet name="Limpieza" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Pearson" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="T6.2 Radio RQD" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="GroupKFold" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="LOOCV-Caserón" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="LOOCV-Caserón métodos" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Importancia" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="Comparación" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="UCS por litología" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="PEP estratos" sheetId="12" state="visible" r:id="rId14"/>
-    <sheet name="Concordancia 1541" sheetId="13" state="visible" r:id="rId15"/>
-    <sheet name="T6.3 Dominios" sheetId="14" state="visible" r:id="rId16"/>
-    <sheet name="T6.4 Ranking" sheetId="15" state="visible" r:id="rId17"/>
-    <sheet name="Bloques" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="DI ventanas" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="GroupKFold" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="LOOCV-Caserón" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="LOOCV-Caserón métodos" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Importancia" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Comparación" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="UCS por litología" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="PEP estratos" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="Concordancia 1541" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="T6.3 Dominios" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="T6.4 Ranking" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="Bloques" sheetId="17" state="visible" r:id="rId19"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="299">
   <si>
     <t xml:space="preserve">Configuración de la corrida final (2026-10-22)</t>
   </si>
@@ -310,6 +311,51 @@
     <t xml:space="preserve">Umbral 1.0 · ventana 14 · 401 combinaciones (400 Dirichlet + convención, semilla 42). Celdas vacías: sin pares suficientes.</t>
   </si>
   <si>
+    <t xml:space="preserve">Sensibilidad del DI al tamaño de ventana (10, 14 y 20 muestras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pozo de referencia PCC_0042_PR01_TH_P20_H12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana [muestras]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana [cm]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registros con DI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% sobre umbral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuatro caserones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pozos sin DI (cortos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picos por 100 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caserón PCC_0042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caserón PCC_1541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caserón PCS_1043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caserón PCS_1059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umbral DI 1.0; pesos calibrados a 5 m; serie depurada (emboquillado y percusión de empate fuera). Picos: eventos sobre el umbral agrupados si están a menos de 0.5 m.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Validación del Random Forest · GroupKFold por pozo (k = 5)</t>
   </si>
   <si>
@@ -638,9 +684,6 @@
   </si>
   <si>
     <t xml:space="preserve">Umbral DI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Picos</t>
   </si>
   <si>
     <t xml:space="preserve">Cruces</t>
@@ -904,9 +947,9 @@
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="0"/>
     <numFmt numFmtId="170" formatCode="\+0.000;\-0.000"/>
-    <numFmt numFmtId="171" formatCode="0.000"/>
-    <numFmt numFmtId="172" formatCode="\+0.0;\-0.0"/>
-    <numFmt numFmtId="173" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="0.0%"/>
+    <numFmt numFmtId="172" formatCode="0.000"/>
+    <numFmt numFmtId="173" formatCode="\+0.0;\-0.0"/>
     <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%"/>
     <numFmt numFmtId="175" formatCode="#,##0.0"/>
   </numFmts>
@@ -1115,6 +1158,14 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="171" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1123,15 +1174,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1147,11 +1190,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1607,6 +1650,156 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="25" t="n">
+        <v>0.2225</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="26" t="n">
+        <v>0.1306</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5" s="25" t="n">
+        <v>0.0494</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>0.0427</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="25" t="n">
+        <v>0.0409</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>0.0156</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>0.0094</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="25" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="26" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="25" t="n">
+        <v>0.323</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" s="26" t="n">
+        <v>29.7</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B18" s="25" t="n">
+        <v>723601</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1621,43 +1814,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>149</v>
+        <v>164</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B3" s="23" t="n">
+        <v>174</v>
+      </c>
+      <c r="B3" s="25" t="n">
         <v>0.184</v>
       </c>
       <c r="C3" s="17" t="n">
         <v>0.136</v>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="25" t="n">
         <v>0.04</v>
       </c>
       <c r="E3" s="14" t="n">
@@ -1666,22 +1859,22 @@
       <c r="F3" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="23" t="n">
+      <c r="G3" s="25" t="n">
         <f aca="false">B3-C3</f>
         <v>0.048</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="B4" s="24" t="n">
+        <v>175</v>
+      </c>
+      <c r="B4" s="26" t="n">
         <v>0.703</v>
       </c>
       <c r="C4" s="19" t="n">
         <v>-0.059</v>
       </c>
-      <c r="D4" s="24" t="n">
+      <c r="D4" s="26" t="n">
         <v>0.222</v>
       </c>
       <c r="E4" s="15" t="n">
@@ -1690,7 +1883,7 @@
       <c r="F4" s="15" t="n">
         <v>3.7</v>
       </c>
-      <c r="G4" s="24" t="n">
+      <c r="G4" s="26" t="n">
         <f aca="false">B4-C4</f>
         <v>0.762</v>
       </c>
@@ -1699,13 +1892,13 @@
       <c r="A5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="25" t="n">
         <v>0.485</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>0.166</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="25" t="n">
         <v>0.189</v>
       </c>
       <c r="E5" s="14" t="n">
@@ -1714,22 +1907,22 @@
       <c r="F5" s="14" t="n">
         <v>3.6</v>
       </c>
-      <c r="G5" s="23" t="n">
+      <c r="G5" s="25" t="n">
         <f aca="false">B5-C5</f>
         <v>0.319</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="B6" s="24" t="n">
+        <v>176</v>
+      </c>
+      <c r="B6" s="26" t="n">
         <v>0.594</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>0.147</v>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="26" t="n">
         <v>0.227</v>
       </c>
       <c r="E6" s="15" t="n">
@@ -1738,22 +1931,22 @@
       <c r="F6" s="15" t="n">
         <v>4.1</v>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="26" t="n">
         <f aca="false">B6-C6</f>
         <v>0.447</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="B7" s="23" t="n">
+        <v>177</v>
+      </c>
+      <c r="B7" s="25" t="n">
         <v>0.492</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>0.088</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="25" t="n">
         <v>0.214</v>
       </c>
       <c r="E7" s="14" t="n">
@@ -1762,14 +1955,14 @@
       <c r="F7" s="14" t="n">
         <v>2.9</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="25" t="n">
         <f aca="false">B7-C7</f>
         <v>0.404</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -1783,7 +1976,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1801,7 +1994,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1815,16 +2008,16 @@
         <v>66</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1846,7 +2039,7 @@
       <c r="F3" s="14" t="n">
         <v>155.7</v>
       </c>
-      <c r="G3" s="25" t="n">
+      <c r="G3" s="27" t="n">
         <f aca="false">E3-C3</f>
         <v>73</v>
       </c>
@@ -1870,7 +2063,7 @@
       <c r="F4" s="15" t="n">
         <v>160.4</v>
       </c>
-      <c r="G4" s="26" t="n">
+      <c r="G4" s="28" t="n">
         <f aca="false">E4-C4</f>
         <v>43.1</v>
       </c>
@@ -1894,7 +2087,7 @@
       <c r="F5" s="14" t="n">
         <v>164.3</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="27" t="n">
         <f aca="false">E5-C5</f>
         <v>9.5</v>
       </c>
@@ -1918,33 +2111,33 @@
       <c r="F6" s="15" t="n">
         <v>177.3</v>
       </c>
-      <c r="G6" s="26" t="n">
+      <c r="G6" s="28" t="n">
         <f aca="false">E6-C6</f>
         <v>-12.7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>735674</v>
@@ -1958,7 +2151,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>150985</v>
@@ -1981,7 +2174,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1998,7 +2191,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2009,19 +2202,19 @@
         <v>66</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2032,7 +2225,7 @@
         <v>128.1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>153</v>
@@ -2040,10 +2233,10 @@
       <c r="E3" s="14" t="n">
         <v>237.149038176504</v>
       </c>
-      <c r="F3" s="23" t="n">
+      <c r="F3" s="25" t="n">
         <v>0.421371709033684</v>
       </c>
-      <c r="G3" s="23" t="n">
+      <c r="G3" s="25" t="n">
         <v>0.844</v>
       </c>
     </row>
@@ -2055,7 +2248,7 @@
         <v>128.1</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>331</v>
@@ -2063,10 +2256,10 @@
       <c r="E4" s="15" t="n">
         <v>263.852272427441</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="26" t="n">
         <v>0.395598425949618</v>
       </c>
-      <c r="G4" s="24" t="n">
+      <c r="G4" s="26" t="n">
         <v>0.788</v>
       </c>
     </row>
@@ -2078,7 +2271,7 @@
         <v>128.1</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>1439</v>
@@ -2086,10 +2279,10 @@
       <c r="E5" s="14" t="n">
         <v>342.535483318491</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="25" t="n">
         <v>0.474310507926838</v>
       </c>
-      <c r="G5" s="23" t="n">
+      <c r="G5" s="25" t="n">
         <v>0.624</v>
       </c>
     </row>
@@ -2101,7 +2294,7 @@
         <v>128.1</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>3303</v>
@@ -2109,10 +2302,10 @@
       <c r="E6" s="15" t="n">
         <v>332.586897951087</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="26" t="n">
         <v>0.413680474209057</v>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="26" t="n">
         <v>0.681</v>
       </c>
     </row>
@@ -2124,7 +2317,7 @@
         <v>128.1</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>6204</v>
@@ -2132,10 +2325,10 @@
       <c r="E7" s="14" t="n">
         <v>371.261248369199</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="25" t="n">
         <v>0.375096773281548</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="25" t="n">
         <v>0.646</v>
       </c>
     </row>
@@ -2147,7 +2340,7 @@
         <v>128.1</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>4488</v>
@@ -2155,10 +2348,10 @@
       <c r="E8" s="15" t="n">
         <v>359.26123899181</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="26" t="n">
         <v>0.358362457170613</v>
       </c>
-      <c r="G8" s="24" t="n">
+      <c r="G8" s="26" t="n">
         <v>0.681</v>
       </c>
     </row>
@@ -2170,7 +2363,7 @@
         <v>128.1</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>8306</v>
@@ -2178,10 +2371,10 @@
       <c r="E9" s="14" t="n">
         <v>327.986036083822</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="25" t="n">
         <v>0.313833984063358</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="25" t="n">
         <v>0.817</v>
       </c>
     </row>
@@ -2193,7 +2386,7 @@
         <v>128.1</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="D10" s="10" t="n">
         <v>7523</v>
@@ -2201,10 +2394,10 @@
       <c r="E10" s="15" t="n">
         <v>325.614844207006</v>
       </c>
-      <c r="F10" s="24" t="n">
+      <c r="F10" s="26" t="n">
         <v>0.299534802737164</v>
       </c>
-      <c r="G10" s="24" t="n">
+      <c r="G10" s="26" t="n">
         <v>0.832</v>
       </c>
     </row>
@@ -2216,7 +2409,7 @@
         <v>128.1</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>17670</v>
@@ -2224,10 +2417,10 @@
       <c r="E11" s="14" t="n">
         <v>332.288926533558</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="25" t="n">
         <v>0.247739838365748</v>
       </c>
-      <c r="G11" s="23" t="n">
+      <c r="G11" s="25" t="n">
         <v>0.881</v>
       </c>
     </row>
@@ -2239,7 +2432,7 @@
         <v>128.1</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="D12" s="10" t="n">
         <v>17807</v>
@@ -2247,10 +2440,10 @@
       <c r="E12" s="15" t="n">
         <v>323.793416204548</v>
       </c>
-      <c r="F12" s="24" t="n">
+      <c r="F12" s="26" t="n">
         <v>0.24797376843445</v>
       </c>
-      <c r="G12" s="24" t="n">
+      <c r="G12" s="26" t="n">
         <v>0.934</v>
       </c>
     </row>
@@ -2262,7 +2455,7 @@
         <v>128.1</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>8826</v>
@@ -2270,10 +2463,10 @@
       <c r="E13" s="14" t="n">
         <v>309.589047051587</v>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F13" s="25" t="n">
         <v>0.262267410701288</v>
       </c>
-      <c r="G13" s="23" t="n">
+      <c r="G13" s="25" t="n">
         <v>0.998</v>
       </c>
     </row>
@@ -2285,7 +2478,7 @@
         <v>128.1</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>17252</v>
@@ -2293,10 +2486,10 @@
       <c r="E14" s="15" t="n">
         <v>305.891885977378</v>
       </c>
-      <c r="F14" s="24" t="n">
+      <c r="F14" s="26" t="n">
         <v>0.244693269104311</v>
       </c>
-      <c r="G14" s="24" t="n">
+      <c r="G14" s="26" t="n">
         <v>1.072</v>
       </c>
     </row>
@@ -2308,7 +2501,7 @@
         <v>128.1</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>59398</v>
@@ -2316,10 +2509,10 @@
       <c r="E15" s="14" t="n">
         <v>322.195476882075</v>
       </c>
-      <c r="F15" s="23" t="n">
+      <c r="F15" s="25" t="n">
         <v>0.211716081126312</v>
       </c>
-      <c r="G15" s="23" t="n">
+      <c r="G15" s="25" t="n">
         <v>1.068</v>
       </c>
     </row>
@@ -2331,7 +2524,7 @@
         <v>128.1</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D16" s="10" t="n">
         <v>71391</v>
@@ -2339,10 +2532,10 @@
       <c r="E16" s="15" t="n">
         <v>348.548507137548</v>
       </c>
-      <c r="F16" s="24" t="n">
+      <c r="F16" s="26" t="n">
         <v>0.194802604846406</v>
       </c>
-      <c r="G16" s="24" t="n">
+      <c r="G16" s="26" t="n">
         <v>0.998</v>
       </c>
     </row>
@@ -2354,7 +2547,7 @@
         <v>111.5</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>40</v>
@@ -2362,10 +2555,10 @@
       <c r="E17" s="14" t="n">
         <v>490.002845904483</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="25" t="n">
         <v>0.324403964150271</v>
       </c>
-      <c r="G17" s="23" t="n">
+      <c r="G17" s="25" t="n">
         <v>0.434</v>
       </c>
     </row>
@@ -2377,7 +2570,7 @@
         <v>111.5</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="D18" s="10" t="n">
         <v>54</v>
@@ -2385,10 +2578,10 @@
       <c r="E18" s="15" t="n">
         <v>557.009518832555</v>
       </c>
-      <c r="F18" s="24" t="n">
+      <c r="F18" s="26" t="n">
         <v>0.346955435487386</v>
       </c>
-      <c r="G18" s="24" t="n">
+      <c r="G18" s="26" t="n">
         <v>0.389</v>
       </c>
     </row>
@@ -2400,7 +2593,7 @@
         <v>111.5</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>106</v>
@@ -2408,10 +2601,10 @@
       <c r="E19" s="14" t="n">
         <v>617.815066800507</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="F19" s="25" t="n">
         <v>0.341841031580977</v>
       </c>
-      <c r="G19" s="23" t="n">
+      <c r="G19" s="25" t="n">
         <v>0.3715</v>
       </c>
     </row>
@@ -2423,7 +2616,7 @@
         <v>111.5</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="D20" s="10" t="n">
         <v>76</v>
@@ -2431,10 +2624,10 @@
       <c r="E20" s="15" t="n">
         <v>506.253719656951</v>
       </c>
-      <c r="F20" s="24" t="n">
+      <c r="F20" s="26" t="n">
         <v>0.428586427145581</v>
       </c>
-      <c r="G20" s="24" t="n">
+      <c r="G20" s="26" t="n">
         <v>0.4995</v>
       </c>
     </row>
@@ -2446,7 +2639,7 @@
         <v>111.5</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>116</v>
@@ -2454,10 +2647,10 @@
       <c r="E21" s="14" t="n">
         <v>390.702302862281</v>
       </c>
-      <c r="F21" s="23" t="n">
+      <c r="F21" s="25" t="n">
         <v>0.272872915686073</v>
       </c>
-      <c r="G21" s="23" t="n">
+      <c r="G21" s="25" t="n">
         <v>0.681</v>
       </c>
     </row>
@@ -2469,7 +2662,7 @@
         <v>111.5</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="D22" s="10" t="n">
         <v>292</v>
@@ -2477,10 +2670,10 @@
       <c r="E22" s="15" t="n">
         <v>400.704367313656</v>
       </c>
-      <c r="F22" s="24" t="n">
+      <c r="F22" s="26" t="n">
         <v>0.311962405709972</v>
       </c>
-      <c r="G22" s="24" t="n">
+      <c r="G22" s="26" t="n">
         <v>0.713</v>
       </c>
     </row>
@@ -2492,7 +2685,7 @@
         <v>111.5</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="D23" s="7" t="n">
         <v>3030</v>
@@ -2500,10 +2693,10 @@
       <c r="E23" s="14" t="n">
         <v>480.245389310267</v>
       </c>
-      <c r="F23" s="23" t="n">
+      <c r="F23" s="25" t="n">
         <v>0.279693777433975</v>
       </c>
-      <c r="G23" s="23" t="n">
+      <c r="G23" s="25" t="n">
         <v>0.599</v>
       </c>
     </row>
@@ -2515,7 +2708,7 @@
         <v>111.5</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="D24" s="10" t="n">
         <v>2672</v>
@@ -2523,10 +2716,10 @@
       <c r="E24" s="15" t="n">
         <v>471.621622585155</v>
       </c>
-      <c r="F24" s="24" t="n">
+      <c r="F24" s="26" t="n">
         <v>0.26316126226668</v>
       </c>
-      <c r="G24" s="24" t="n">
+      <c r="G24" s="26" t="n">
         <v>0.623</v>
       </c>
     </row>
@@ -2538,7 +2731,7 @@
         <v>111.5</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>2282</v>
@@ -2546,10 +2739,10 @@
       <c r="E25" s="14" t="n">
         <v>430.282771322748</v>
       </c>
-      <c r="F25" s="23" t="n">
+      <c r="F25" s="25" t="n">
         <v>0.210061338770437</v>
       </c>
-      <c r="G25" s="23" t="n">
+      <c r="G25" s="25" t="n">
         <v>0.713</v>
       </c>
     </row>
@@ -2561,7 +2754,7 @@
         <v>111.5</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="D26" s="10" t="n">
         <v>1979</v>
@@ -2569,10 +2762,10 @@
       <c r="E26" s="15" t="n">
         <v>432.658707257502</v>
       </c>
-      <c r="F26" s="24" t="n">
+      <c r="F26" s="26" t="n">
         <v>0.19553590386331</v>
       </c>
-      <c r="G26" s="24" t="n">
+      <c r="G26" s="26" t="n">
         <v>0.737</v>
       </c>
     </row>
@@ -2584,7 +2777,7 @@
         <v>111.5</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>1986</v>
@@ -2592,10 +2785,10 @@
       <c r="E27" s="14" t="n">
         <v>408.695485284908</v>
       </c>
-      <c r="F27" s="23" t="n">
+      <c r="F27" s="25" t="n">
         <v>0.189134161189736</v>
       </c>
-      <c r="G27" s="23" t="n">
+      <c r="G27" s="25" t="n">
         <v>0.831</v>
       </c>
     </row>
@@ -2607,7 +2800,7 @@
         <v>111.5</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="D28" s="10" t="n">
         <v>3550</v>
@@ -2615,10 +2808,10 @@
       <c r="E28" s="15" t="n">
         <v>478.759322570568</v>
       </c>
-      <c r="F28" s="24" t="n">
+      <c r="F28" s="26" t="n">
         <v>0.175511683493541</v>
       </c>
-      <c r="G28" s="24" t="n">
+      <c r="G28" s="26" t="n">
         <v>0.739</v>
       </c>
     </row>
@@ -2630,7 +2823,7 @@
         <v>111.5</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>603</v>
@@ -2638,10 +2831,10 @@
       <c r="E29" s="14" t="n">
         <v>454.142856536525</v>
       </c>
-      <c r="F29" s="23" t="n">
+      <c r="F29" s="25" t="n">
         <v>0.189662936155716</v>
       </c>
-      <c r="G29" s="23" t="n">
+      <c r="G29" s="25" t="n">
         <v>0.748</v>
       </c>
     </row>
@@ -2653,7 +2846,7 @@
         <v>180</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="D30" s="10" t="n">
         <v>126</v>
@@ -2661,10 +2854,10 @@
       <c r="E30" s="15" t="n">
         <v>234.369944504969</v>
       </c>
-      <c r="F30" s="24" t="n">
+      <c r="F30" s="26" t="n">
         <v>0.42473313654433</v>
       </c>
-      <c r="G30" s="24" t="n">
+      <c r="G30" s="26" t="n">
         <v>0.8795</v>
       </c>
     </row>
@@ -2676,7 +2869,7 @@
         <v>180</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>282</v>
@@ -2684,10 +2877,10 @@
       <c r="E31" s="14" t="n">
         <v>258.058823253413</v>
       </c>
-      <c r="F31" s="23" t="n">
+      <c r="F31" s="25" t="n">
         <v>0.428103876319314</v>
       </c>
-      <c r="G31" s="23" t="n">
+      <c r="G31" s="25" t="n">
         <v>0.8315</v>
       </c>
     </row>
@@ -2699,7 +2892,7 @@
         <v>180</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="D32" s="10" t="n">
         <v>738</v>
@@ -2707,10 +2900,10 @@
       <c r="E32" s="15" t="n">
         <v>346.205203757051</v>
       </c>
-      <c r="F32" s="24" t="n">
+      <c r="F32" s="26" t="n">
         <v>0.597428034253832</v>
       </c>
-      <c r="G32" s="24" t="n">
+      <c r="G32" s="26" t="n">
         <v>0.674</v>
       </c>
     </row>
@@ -2722,7 +2915,7 @@
         <v>180</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="D33" s="7" t="n">
         <v>1542</v>
@@ -2730,10 +2923,10 @@
       <c r="E33" s="14" t="n">
         <v>367.443491716508</v>
       </c>
-      <c r="F33" s="23" t="n">
+      <c r="F33" s="25" t="n">
         <v>0.534254422933826</v>
       </c>
-      <c r="G33" s="23" t="n">
+      <c r="G33" s="25" t="n">
         <v>0.65</v>
       </c>
     </row>
@@ -2745,7 +2938,7 @@
         <v>180</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="D34" s="10" t="n">
         <v>7341</v>
@@ -2753,10 +2946,10 @@
       <c r="E34" s="15" t="n">
         <v>444.381782084531</v>
       </c>
-      <c r="F34" s="24" t="n">
+      <c r="F34" s="26" t="n">
         <v>0.369032113926087</v>
       </c>
-      <c r="G34" s="24" t="n">
+      <c r="G34" s="26" t="n">
         <v>0.554</v>
       </c>
     </row>
@@ -2768,7 +2961,7 @@
         <v>180</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>7554</v>
@@ -2776,10 +2969,10 @@
       <c r="E35" s="14" t="n">
         <v>414.249439913248</v>
       </c>
-      <c r="F35" s="23" t="n">
+      <c r="F35" s="25" t="n">
         <v>0.364801845435549</v>
       </c>
-      <c r="G35" s="23" t="n">
+      <c r="G35" s="25" t="n">
         <v>0.599</v>
       </c>
     </row>
@@ -2791,7 +2984,7 @@
         <v>180</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>11164</v>
@@ -2799,10 +2992,10 @@
       <c r="E36" s="15" t="n">
         <v>371.956160266194</v>
       </c>
-      <c r="F36" s="24" t="n">
+      <c r="F36" s="26" t="n">
         <v>0.285560228063442</v>
       </c>
-      <c r="G36" s="24" t="n">
+      <c r="G36" s="26" t="n">
         <v>0.749</v>
       </c>
     </row>
@@ -2814,7 +3007,7 @@
         <v>180</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="D37" s="7" t="n">
         <v>11833</v>
@@ -2822,10 +3015,10 @@
       <c r="E37" s="14" t="n">
         <v>361.053475453137</v>
       </c>
-      <c r="F37" s="23" t="n">
+      <c r="F37" s="25" t="n">
         <v>0.288288967090207</v>
       </c>
-      <c r="G37" s="23" t="n">
+      <c r="G37" s="25" t="n">
         <v>0.789</v>
       </c>
     </row>
@@ -2837,7 +3030,7 @@
         <v>180</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="D38" s="10" t="n">
         <v>30363</v>
@@ -2845,10 +3038,10 @@
       <c r="E38" s="15" t="n">
         <v>375.914663009718</v>
       </c>
-      <c r="F38" s="24" t="n">
+      <c r="F38" s="26" t="n">
         <v>0.267034079014971</v>
       </c>
-      <c r="G38" s="24" t="n">
+      <c r="G38" s="26" t="n">
         <v>0.788</v>
       </c>
     </row>
@@ -2860,7 +3053,7 @@
         <v>180</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>16372</v>
@@ -2868,10 +3061,10 @@
       <c r="E39" s="14" t="n">
         <v>388.285713767309</v>
       </c>
-      <c r="F39" s="23" t="n">
+      <c r="F39" s="25" t="n">
         <v>0.299879396218285</v>
       </c>
-      <c r="G39" s="23" t="n">
+      <c r="G39" s="25" t="n">
         <v>0.788</v>
       </c>
     </row>
@@ -2883,7 +3076,7 @@
         <v>180</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="D40" s="10" t="n">
         <v>10824</v>
@@ -2891,10 +3084,10 @@
       <c r="E40" s="15" t="n">
         <v>330.755061252211</v>
       </c>
-      <c r="F40" s="24" t="n">
+      <c r="F40" s="26" t="n">
         <v>0.29088489802897</v>
       </c>
-      <c r="G40" s="24" t="n">
+      <c r="G40" s="26" t="n">
         <v>0.998</v>
       </c>
     </row>
@@ -2906,7 +3099,7 @@
         <v>180</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>48445</v>
@@ -2914,10 +3107,10 @@
       <c r="E41" s="14" t="n">
         <v>350.372548658026</v>
       </c>
-      <c r="F41" s="23" t="n">
+      <c r="F41" s="25" t="n">
         <v>0.221604678793535</v>
       </c>
-      <c r="G41" s="23" t="n">
+      <c r="G41" s="25" t="n">
         <v>0.967</v>
       </c>
     </row>
@@ -2929,7 +3122,7 @@
         <v>180</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="D42" s="10" t="n">
         <v>66162</v>
@@ -2937,10 +3130,10 @@
       <c r="E42" s="15" t="n">
         <v>337.243625574617</v>
       </c>
-      <c r="F42" s="24" t="n">
+      <c r="F42" s="26" t="n">
         <v>0.24118899908423</v>
       </c>
-      <c r="G42" s="24" t="n">
+      <c r="G42" s="26" t="n">
         <v>1.033</v>
       </c>
     </row>
@@ -2952,7 +3145,7 @@
         <v>180</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D43" s="7" t="n">
         <v>211422</v>
@@ -2960,10 +3153,10 @@
       <c r="E43" s="14" t="n">
         <v>368.672637127576</v>
       </c>
-      <c r="F43" s="23" t="n">
+      <c r="F43" s="25" t="n">
         <v>0.185374113646284</v>
       </c>
-      <c r="G43" s="23" t="n">
+      <c r="G43" s="25" t="n">
         <v>0.969</v>
       </c>
     </row>
@@ -2975,7 +3168,7 @@
         <v>60</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="D44" s="10" t="n">
         <v>34</v>
@@ -2983,10 +3176,10 @@
       <c r="E44" s="15" t="n">
         <v>209.757971600888</v>
       </c>
-      <c r="F44" s="24" t="n">
+      <c r="F44" s="26" t="n">
         <v>0.517428568469482</v>
       </c>
-      <c r="G44" s="24" t="n">
+      <c r="G44" s="26" t="n">
         <v>1.07</v>
       </c>
     </row>
@@ -2998,7 +3191,7 @@
         <v>60</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="D45" s="7" t="n">
         <v>54</v>
@@ -3006,10 +3199,10 @@
       <c r="E45" s="14" t="n">
         <v>190.795721316447</v>
       </c>
-      <c r="F45" s="23" t="n">
+      <c r="F45" s="25" t="n">
         <v>0.562164373559164</v>
       </c>
-      <c r="G45" s="23" t="n">
+      <c r="G45" s="25" t="n">
         <v>1.153</v>
       </c>
     </row>
@@ -3021,7 +3214,7 @@
         <v>60</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="D46" s="10" t="n">
         <v>410</v>
@@ -3029,10 +3222,10 @@
       <c r="E46" s="15" t="n">
         <v>270.604217215766</v>
       </c>
-      <c r="F46" s="24" t="n">
+      <c r="F46" s="26" t="n">
         <v>0.331366297071089</v>
       </c>
-      <c r="G46" s="24" t="n">
+      <c r="G46" s="26" t="n">
         <v>0.817</v>
       </c>
     </row>
@@ -3044,7 +3237,7 @@
         <v>60</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="D47" s="7" t="n">
         <v>729</v>
@@ -3052,10 +3245,10 @@
       <c r="E47" s="14" t="n">
         <v>288.579800138928</v>
       </c>
-      <c r="F47" s="23" t="n">
+      <c r="F47" s="25" t="n">
         <v>0.388493304716055</v>
       </c>
-      <c r="G47" s="23" t="n">
+      <c r="G47" s="25" t="n">
         <v>0.788</v>
       </c>
     </row>
@@ -3067,7 +3260,7 @@
         <v>60</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="D48" s="10" t="n">
         <v>971</v>
@@ -3075,10 +3268,10 @@
       <c r="E48" s="15" t="n">
         <v>288.974477622999</v>
       </c>
-      <c r="F48" s="24" t="n">
+      <c r="F48" s="26" t="n">
         <v>0.356738284292291</v>
       </c>
-      <c r="G48" s="24" t="n">
+      <c r="G48" s="26" t="n">
         <v>0.832</v>
       </c>
     </row>
@@ -3090,7 +3283,7 @@
         <v>60</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="D49" s="7" t="n">
         <v>980</v>
@@ -3098,10 +3291,10 @@
       <c r="E49" s="14" t="n">
         <v>300.610011720505</v>
       </c>
-      <c r="F49" s="23" t="n">
+      <c r="F49" s="25" t="n">
         <v>0.391610531514125</v>
       </c>
-      <c r="G49" s="23" t="n">
+      <c r="G49" s="25" t="n">
         <v>0.832</v>
       </c>
     </row>
@@ -3113,7 +3306,7 @@
         <v>60</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="D50" s="10" t="n">
         <v>736</v>
@@ -3121,10 +3314,10 @@
       <c r="E50" s="15" t="n">
         <v>277.0931323157</v>
       </c>
-      <c r="F50" s="24" t="n">
+      <c r="F50" s="26" t="n">
         <v>0.388379325521793</v>
       </c>
-      <c r="G50" s="24" t="n">
+      <c r="G50" s="26" t="n">
         <v>0.936</v>
       </c>
     </row>
@@ -3136,7 +3329,7 @@
         <v>60</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="D51" s="7" t="n">
         <v>789</v>
@@ -3144,10 +3337,10 @@
       <c r="E51" s="14" t="n">
         <v>257.340504904265</v>
       </c>
-      <c r="F51" s="23" t="n">
+      <c r="F51" s="25" t="n">
         <v>0.414490242049583</v>
       </c>
-      <c r="G51" s="23" t="n">
+      <c r="G51" s="25" t="n">
         <v>1.069</v>
       </c>
     </row>
@@ -3159,7 +3352,7 @@
         <v>60</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="D52" s="10" t="n">
         <v>4921</v>
@@ -3167,10 +3360,10 @@
       <c r="E52" s="15" t="n">
         <v>305.811440354013</v>
       </c>
-      <c r="F52" s="24" t="n">
+      <c r="F52" s="26" t="n">
         <v>0.284658189345987</v>
       </c>
-      <c r="G52" s="24" t="n">
+      <c r="G52" s="26" t="n">
         <v>0.944</v>
       </c>
     </row>
@@ -3182,7 +3375,7 @@
         <v>60</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="D53" s="7" t="n">
         <v>3689</v>
@@ -3190,10 +3383,10 @@
       <c r="E53" s="14" t="n">
         <v>313.372933560565</v>
       </c>
-      <c r="F53" s="23" t="n">
+      <c r="F53" s="25" t="n">
         <v>0.277362949989555</v>
       </c>
-      <c r="G53" s="23" t="n">
+      <c r="G53" s="25" t="n">
         <v>0.936</v>
       </c>
     </row>
@@ -3205,7 +3398,7 @@
         <v>60</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="D54" s="10" t="n">
         <v>1230</v>
@@ -3213,10 +3406,10 @@
       <c r="E54" s="15" t="n">
         <v>223.615416028833</v>
       </c>
-      <c r="F54" s="24" t="n">
+      <c r="F54" s="26" t="n">
         <v>0.320460196010326</v>
       </c>
-      <c r="G54" s="24" t="n">
+      <c r="G54" s="26" t="n">
         <v>1.408</v>
       </c>
     </row>
@@ -3228,7 +3421,7 @@
         <v>60</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="D55" s="7" t="n">
         <v>6302</v>
@@ -3236,10 +3429,10 @@
       <c r="E55" s="14" t="n">
         <v>283.289930309644</v>
       </c>
-      <c r="F55" s="23" t="n">
+      <c r="F55" s="25" t="n">
         <v>0.242946629747541</v>
       </c>
-      <c r="G55" s="23" t="n">
+      <c r="G55" s="25" t="n">
         <v>1.152</v>
       </c>
     </row>
@@ -3251,7 +3444,7 @@
         <v>60</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="D56" s="10" t="n">
         <v>7892</v>
@@ -3259,10 +3452,10 @@
       <c r="E56" s="15" t="n">
         <v>274.58134357701</v>
       </c>
-      <c r="F56" s="24" t="n">
+      <c r="F56" s="26" t="n">
         <v>0.259383834173968</v>
       </c>
-      <c r="G56" s="24" t="n">
+      <c r="G56" s="26" t="n">
         <v>1.233</v>
       </c>
     </row>
@@ -3274,7 +3467,7 @@
         <v>60</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D57" s="7" t="n">
         <v>24255</v>
@@ -3282,29 +3475,29 @@
       <c r="E57" s="14" t="n">
         <v>309.786025930318</v>
       </c>
-      <c r="F57" s="23" t="n">
+      <c r="F57" s="25" t="n">
         <v>0.182065821735189</v>
       </c>
-      <c r="G57" s="23" t="n">
+      <c r="G57" s="25" t="n">
         <v>1.109</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="B61" s="17" t="n">
         <v>0.203</v>
@@ -3312,7 +3505,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="B62" s="19" t="n">
         <v>-0.904</v>
@@ -3328,7 +3521,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -3342,7 +3535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3361,30 +3554,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>201</v>
+        <v>96</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3397,16 +3590,16 @@
       <c r="C3" s="7" t="n">
         <v>415</v>
       </c>
-      <c r="D3" s="27" t="n">
+      <c r="D3" s="20" t="n">
         <v>0.521885521885522</v>
       </c>
-      <c r="E3" s="27" t="n">
+      <c r="E3" s="20" t="n">
         <v>0.407228915662651</v>
       </c>
-      <c r="F3" s="27" t="n">
+      <c r="F3" s="20" t="n">
         <v>0.543097643097643</v>
       </c>
-      <c r="G3" s="28" t="n">
+      <c r="G3" s="29" t="n">
         <f aca="false">D3-F3</f>
         <v>-0.0212121212121211</v>
       </c>
@@ -3421,13 +3614,13 @@
       <c r="C4" s="10" t="n">
         <v>415</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="D4" s="21" t="n">
         <v>0.580853816300129</v>
       </c>
-      <c r="E4" s="29" t="n">
+      <c r="E4" s="21" t="n">
         <v>0.727710843373494</v>
       </c>
-      <c r="F4" s="29" t="n">
+      <c r="F4" s="21" t="n">
         <v>0.519879258300992</v>
       </c>
       <c r="G4" s="30" t="n">
@@ -3445,16 +3638,16 @@
       <c r="C5" s="7" t="n">
         <v>415</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="20" t="n">
         <v>0.58030303030303</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="20" t="n">
         <v>0.927710843373494</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="20" t="n">
         <v>0.526414141414141</v>
       </c>
-      <c r="G5" s="28" t="n">
+      <c r="G5" s="29" t="n">
         <f aca="false">D5-F5</f>
         <v>0.0538888888888889</v>
       </c>
@@ -3469,13 +3662,13 @@
       <c r="C6" s="10" t="n">
         <v>415</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="21" t="n">
         <v>0.514166666666667</v>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="21" t="n">
         <v>0.857831325301205</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="21" t="n">
         <v>0.525722222222222</v>
       </c>
       <c r="G6" s="30" t="n">
@@ -3493,16 +3686,16 @@
       <c r="C7" s="7" t="n">
         <v>415</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="20" t="n">
         <v>0.516237402015678</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="20" t="n">
         <v>0.734939759036145</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="20" t="n">
         <v>0.522471071295259</v>
       </c>
-      <c r="G7" s="28" t="n">
+      <c r="G7" s="29" t="n">
         <f aca="false">D7-F7</f>
         <v>-0.00623366927958191</v>
       </c>
@@ -3517,13 +3710,13 @@
       <c r="C8" s="10" t="n">
         <v>415</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="21" t="n">
         <v>0.524752475247525</v>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="21" t="n">
         <v>0.563855421686747</v>
       </c>
-      <c r="F8" s="29" t="n">
+      <c r="F8" s="21" t="n">
         <v>0.52019801980198</v>
       </c>
       <c r="G8" s="30" t="n">
@@ -3541,16 +3734,16 @@
       <c r="C9" s="7" t="n">
         <v>415</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="20" t="n">
         <v>0.541139240506329</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="20" t="n">
         <v>0.414457831325301</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="20" t="n">
         <v>0.517405063291139</v>
       </c>
-      <c r="G9" s="28" t="n">
+      <c r="G9" s="29" t="n">
         <f aca="false">D9-F9</f>
         <v>0.02373417721519</v>
       </c>
@@ -3565,13 +3758,13 @@
       <c r="C10" s="10" t="n">
         <v>415</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="21" t="n">
         <v>0.443820224719101</v>
       </c>
-      <c r="E10" s="29" t="n">
+      <c r="E10" s="21" t="n">
         <v>0.214457831325301</v>
       </c>
-      <c r="F10" s="29" t="n">
+      <c r="F10" s="21" t="n">
         <v>0.498689138576779</v>
       </c>
       <c r="G10" s="30" t="n">
@@ -3581,20 +3774,20 @@
     </row>
     <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>201</v>
+        <v>96</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>1320</v>
@@ -3602,7 +3795,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="B15" s="32" t="n">
         <v>-0.0758083333333332</v>
@@ -3610,7 +3803,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="B16" s="34" t="n">
         <v>0.152</v>
@@ -3618,7 +3811,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="B17" s="9" t="n">
         <v>5.46420883724733</v>
@@ -3635,7 +3828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3653,46 +3846,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>164.932209858122</v>
       </c>
-      <c r="E3" s="23" t="n">
+      <c r="E3" s="25" t="n">
         <v>0.624956799262139</v>
       </c>
       <c r="F3" s="7" t="n">
@@ -3704,18 +3897,18 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D4" s="15" t="n">
         <v>138.496561143358</v>
       </c>
-      <c r="E4" s="24" t="n">
+      <c r="E4" s="26" t="n">
         <v>0.701199959240213</v>
       </c>
       <c r="F4" s="10" t="n">
@@ -3727,18 +3920,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>134.789098647061</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="25" t="n">
         <v>0.873490925570658</v>
       </c>
       <c r="F5" s="7" t="n">
@@ -3750,18 +3943,18 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>154.123768904038</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="26" t="n">
         <v>1.20733220807777</v>
       </c>
       <c r="F6" s="10" t="n">
@@ -3773,18 +3966,18 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>137.155726282</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="25" t="n">
         <v>0.619054363908438</v>
       </c>
       <c r="F7" s="7" t="n">
@@ -3796,18 +3989,18 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>139.393544557154</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="26" t="n">
         <v>0.729862070803117</v>
       </c>
       <c r="F8" s="10" t="n">
@@ -3819,18 +4012,18 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>153.727676276695</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="25" t="n">
         <v>0.633670922155736</v>
       </c>
       <c r="F9" s="7" t="n">
@@ -3842,18 +4035,18 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>168.41475157952</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="E10" s="26" t="n">
         <v>0.562630038147136</v>
       </c>
       <c r="F10" s="10" t="n">
@@ -3865,18 +4058,18 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>144.172700603197</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="25" t="n">
         <v>1.25329485213606</v>
       </c>
       <c r="F11" s="7" t="n">
@@ -3888,18 +4081,18 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>159.684160752595</v>
       </c>
-      <c r="E12" s="24" t="n">
+      <c r="E12" s="26" t="n">
         <v>0.654783033634757</v>
       </c>
       <c r="F12" s="10" t="n">
@@ -3911,18 +4104,18 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>167.800529418651</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="25" t="n">
         <v>0.627988751299209</v>
       </c>
       <c r="F13" s="7" t="n">
@@ -3934,18 +4127,18 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>124.601455398543</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="26" t="n">
         <v>0.82350210956101</v>
       </c>
       <c r="F14" s="10" t="n">
@@ -3957,18 +4150,18 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>119.768508894793</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="25" t="n">
         <v>0.778168169952817</v>
       </c>
       <c r="F15" s="7" t="n">
@@ -3980,18 +4173,18 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>224</v>
-      </c>
       <c r="C16" s="4" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>119.704137883813</v>
       </c>
-      <c r="E16" s="24" t="n">
+      <c r="E16" s="26" t="n">
         <v>0.596968473291783</v>
       </c>
       <c r="F16" s="10" t="n">
@@ -4003,18 +4196,18 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>158.678228976082</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="25" t="n">
         <v>0.831387540875796</v>
       </c>
       <c r="F17" s="7" t="n">
@@ -4026,7 +4219,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -4040,7 +4233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4060,45 +4253,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>34</v>
@@ -4106,7 +4299,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="B3" s="16" t="n">
         <v>1</v>
@@ -4132,11 +4325,11 @@
       <c r="I3" s="16" t="n">
         <v>500.540267735832</v>
       </c>
-      <c r="J3" s="23" t="n">
+      <c r="J3" s="25" t="n">
         <v>0.0048</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="L3" s="14" t="n">
         <v>18.033</v>
@@ -4147,7 +4340,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>2</v>
@@ -4173,11 +4366,11 @@
       <c r="I4" s="18" t="n">
         <v>373.165042543947</v>
       </c>
-      <c r="J4" s="24" t="n">
+      <c r="J4" s="26" t="n">
         <v>0.0095</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="L4" s="15" t="n">
         <v>23.376</v>
@@ -4188,7 +4381,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>3</v>
@@ -4214,11 +4407,11 @@
       <c r="I5" s="16" t="n">
         <v>402.175669000924</v>
       </c>
-      <c r="J5" s="23" t="n">
+      <c r="J5" s="25" t="n">
         <v>0.0117</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="L5" s="14" t="n">
         <v>10.993</v>
@@ -4229,7 +4422,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>4</v>
@@ -4255,11 +4448,11 @@
       <c r="I6" s="18" t="n">
         <v>400.204833233857</v>
       </c>
-      <c r="J6" s="24" t="n">
+      <c r="J6" s="26" t="n">
         <v>0.0128</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="L6" s="15" t="n">
         <v>28.854</v>
@@ -4270,7 +4463,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>5</v>
@@ -4296,11 +4489,11 @@
       <c r="I7" s="16" t="n">
         <v>325.995300891542</v>
       </c>
-      <c r="J7" s="23" t="n">
+      <c r="J7" s="25" t="n">
         <v>0.0172</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="L7" s="14" t="n">
         <v>17.351</v>
@@ -4311,7 +4504,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>1</v>
@@ -4337,11 +4530,11 @@
       <c r="I8" s="18" t="n">
         <v>162.332346613696</v>
       </c>
-      <c r="J8" s="24" t="n">
+      <c r="J8" s="26" t="n">
         <v>0.1651</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="L8" s="15" t="n">
         <v>20.324</v>
@@ -4352,7 +4545,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>2</v>
@@ -4378,11 +4571,11 @@
       <c r="I9" s="16" t="n">
         <v>166.827549144259</v>
       </c>
-      <c r="J9" s="23" t="n">
+      <c r="J9" s="25" t="n">
         <v>0.2719</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="L9" s="14" t="n">
         <v>26.594</v>
@@ -4393,7 +4586,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>3</v>
@@ -4419,11 +4612,11 @@
       <c r="I10" s="18" t="n">
         <v>167.32673415805</v>
       </c>
-      <c r="J10" s="24" t="n">
+      <c r="J10" s="26" t="n">
         <v>0.0715</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>19.494</v>
@@ -4434,7 +4627,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>4</v>
@@ -4460,11 +4653,11 @@
       <c r="I11" s="16" t="n">
         <v>167.397432996347</v>
       </c>
-      <c r="J11" s="23" t="n">
+      <c r="J11" s="25" t="n">
         <v>0.0977</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="L11" s="14" t="n">
         <v>18.798</v>
@@ -4475,7 +4668,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>5</v>
@@ -4501,11 +4694,11 @@
       <c r="I12" s="18" t="n">
         <v>178.524281693897</v>
       </c>
-      <c r="J12" s="24" t="n">
+      <c r="J12" s="26" t="n">
         <v>0.1226</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="L12" s="15" t="n">
         <v>20.774</v>
@@ -4516,7 +4709,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>1</v>
@@ -4542,11 +4735,11 @@
       <c r="I13" s="16" t="n">
         <v>178.524281693897</v>
       </c>
-      <c r="J13" s="23" t="n">
+      <c r="J13" s="25" t="n">
         <v>0.1226</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="L13" s="14" t="n">
         <v>20.774</v>
@@ -4557,7 +4750,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B14" s="18" t="n">
         <v>2</v>
@@ -4583,11 +4776,11 @@
       <c r="I14" s="18" t="n">
         <v>162.332346613696</v>
       </c>
-      <c r="J14" s="24" t="n">
+      <c r="J14" s="26" t="n">
         <v>0.1651</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="L14" s="15" t="n">
         <v>20.324</v>
@@ -4598,7 +4791,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>3</v>
@@ -4624,11 +4817,11 @@
       <c r="I15" s="16" t="n">
         <v>215.518963920522</v>
       </c>
-      <c r="J15" s="23" t="n">
+      <c r="J15" s="25" t="n">
         <v>0.1055</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="L15" s="14" t="n">
         <v>28.608</v>
@@ -4639,7 +4832,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>4</v>
@@ -4665,11 +4858,11 @@
       <c r="I16" s="18" t="n">
         <v>185.890821831519</v>
       </c>
-      <c r="J16" s="24" t="n">
+      <c r="J16" s="26" t="n">
         <v>0.0952</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="L16" s="15" t="n">
         <v>20.049</v>
@@ -4680,7 +4873,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>5</v>
@@ -4706,11 +4899,11 @@
       <c r="I17" s="16" t="n">
         <v>193.035955279126</v>
       </c>
-      <c r="J17" s="23" t="n">
+      <c r="J17" s="25" t="n">
         <v>0.0423</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="L17" s="14" t="n">
         <v>28.47</v>
@@ -4730,7 +4923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4746,7 +4939,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4754,13 +4947,13 @@
         <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4773,7 +4966,7 @@
       <c r="C3" s="7" t="n">
         <v>424184</v>
       </c>
-      <c r="D3" s="27" t="n">
+      <c r="D3" s="20" t="n">
         <v>0.3172</v>
       </c>
     </row>
@@ -4787,7 +4980,7 @@
       <c r="C4" s="10" t="n">
         <v>176898</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="D4" s="21" t="n">
         <v>0.2555</v>
       </c>
     </row>
@@ -4801,7 +4994,7 @@
       <c r="C5" s="7" t="n">
         <v>141577</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="20" t="n">
         <v>0.233</v>
       </c>
     </row>
@@ -4815,7 +5008,7 @@
       <c r="C6" s="10" t="n">
         <v>126768</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="21" t="n">
         <v>0.2266</v>
       </c>
     </row>
@@ -4834,7 +5027,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>2</v>
@@ -4842,7 +5035,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>233015.6</v>
@@ -4850,15 +5043,15 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="B11" s="29" t="n">
+        <v>286</v>
+      </c>
+      <c r="B11" s="21" t="n">
         <v>0.085</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
       <c r="B12" s="35" t="n">
         <v>0.73</v>
@@ -4866,7 +5059,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="B13" s="36" t="n">
         <v>154.4</v>
@@ -4874,7 +5067,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="B14" s="35" t="n">
         <v>130.9</v>
@@ -4882,7 +5075,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="B15" s="36" t="n">
         <v>170.2</v>
@@ -4890,26 +5083,26 @@
     </row>
     <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
       <c r="C19" s="7" t="n">
         <v>1159</v>
@@ -4917,10 +5110,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>13651</v>
@@ -4928,10 +5121,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>103</v>
@@ -4939,7 +5132,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>
@@ -6061,13 +6254,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6075,162 +6271,626 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B4" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>0.1524</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>0.1717</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>0.1911</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>144720</v>
-      </c>
-      <c r="C3" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" s="17" t="n">
-        <v>0.273</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>29.06</v>
-      </c>
-      <c r="F3" s="17" t="n">
-        <v>0.524</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B4" s="10" t="n">
-        <v>144720</v>
-      </c>
-      <c r="C4" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" s="19" t="n">
-        <v>0.325</v>
-      </c>
-      <c r="E4" s="9" t="n">
-        <v>29.87</v>
-      </c>
-      <c r="F4" s="19" t="n">
-        <v>0.597</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="E9" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>144721</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" s="17" t="n">
-        <v>0.273</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="F5" s="17" t="n">
-        <v>0.557</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="H9" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>928</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>885030</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>8338</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>41.17</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>0.1505</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>928</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>885030</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>7870</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>38.86</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <v>0.1703</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>928</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>884977</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>7218</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>35.64</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="10" t="n">
-        <v>144721</v>
-      </c>
-      <c r="C6" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="19" t="n">
-        <v>0.297</v>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>28.93</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>0.573</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>436</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>434091</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>4280</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>0.1229</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>436</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>434091</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>3873</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>39.18</v>
+      </c>
+      <c r="H17" s="21" t="n">
+        <v>0.1407</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>436</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>434074</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>3433</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>34.73</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>0.1625</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>144719</v>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="17" t="n">
-        <v>0.281</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>32.01</v>
-      </c>
-      <c r="F7" s="17" t="n">
-        <v>0.567</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>237</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>178452</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>1409</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>33.81</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>0.2367</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>237</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>178452</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>1594</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="H23" s="21" t="n">
+        <v>0.2612</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>237</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>178416</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>39.59</v>
+      </c>
+      <c r="H24" s="20" t="n">
+        <v>0.2893</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="20" t="n">
-        <f aca="false">AVERAGE(D3:D7)</f>
-        <v>0.2898</v>
-      </c>
-      <c r="E8" s="21" t="n">
-        <f aca="false">AVERAGE(E3:E7)</f>
-        <v>30.354</v>
-      </c>
-      <c r="F8" s="20" t="n">
-        <f aca="false">AVERAGE(F3:F7)</f>
-        <v>0.5636</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>143472</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>1452</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>44.77</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <v>0.1243</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B29" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="10" t="n">
+        <v>125</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>143472</v>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>1293</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>39.87</v>
+      </c>
+      <c r="H29" s="21" t="n">
+        <v>0.1417</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>143472</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>1113</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>34.32</v>
+      </c>
+      <c r="H30" s="20" t="n">
+        <v>0.1593</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="22" t="n">
-        <f aca="false">STDEV(D3:D7)</f>
-        <v>0.0219818106624545</v>
-      </c>
-      <c r="E9" s="22" t="n">
-        <f aca="false">STDEV(E3:E7)</f>
-        <v>1.50573237994007</v>
-      </c>
-      <c r="F9" s="22" t="n">
-        <f aca="false">STDEV(F3:F7)</f>
-        <v>0.0265857104475317</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B34" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>129015</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>1197</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>40.47</v>
+      </c>
+      <c r="H34" s="20" t="n">
+        <v>0.1534</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B35" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>130</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="10" t="n">
+        <v>129015</v>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>1110</v>
+      </c>
+      <c r="G35" s="9" t="n">
+        <v>37.53</v>
+      </c>
+      <c r="H35" s="21" t="n">
+        <v>0.1757</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B36" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>129015</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>1022</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>34.56</v>
+      </c>
+      <c r="H36" s="20" t="n">
+        <v>0.2002</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -6253,7 +6913,7 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
@@ -6269,122 +6929,158 @@
         <v>107</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>60</v>
+        <v>113</v>
       </c>
       <c r="B3" s="7" t="n">
-        <v>365414</v>
+        <v>144720</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D3" s="17" t="n">
-        <v>-3.547</v>
+        <v>0.273</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>44.85</v>
+        <v>29.06</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>0.237</v>
+        <v>0.524</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>61</v>
+        <v>114</v>
       </c>
       <c r="B4" s="10" t="n">
-        <v>131053</v>
+        <v>144720</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>-4.138</v>
+        <v>0.325</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>75.89</v>
+        <v>29.87</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>0.049</v>
+        <v>0.597</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="B5" s="7" t="n">
-        <v>122026</v>
+        <v>144721</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>-0.613</v>
+        <v>0.273</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>31.58</v>
+        <v>31.9</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.048</v>
+        <v>0.557</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="B6" s="10" t="n">
-        <v>105108</v>
+        <v>144721</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="19"/>
+        <v>4</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0.297</v>
+      </c>
       <c r="E6" s="9" t="n">
-        <v>49.81</v>
-      </c>
-      <c r="F6" s="19"/>
+        <v>28.93</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.573</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="20" t="n">
-        <f aca="false">AVERAGE(D3:D6)</f>
-        <v>-2.766</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <f aca="false">AVERAGE(E3:E6)</f>
-        <v>50.5325</v>
-      </c>
-      <c r="F7" s="20" t="n">
-        <f aca="false">AVERAGE(F3:F6)</f>
-        <v>0.111333333333333</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>109</v>
+      <c r="A7" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>144719</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>0.567</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <f aca="false">AVERAGE(D3:D7)</f>
+        <v>0.2898</v>
+      </c>
+      <c r="E8" s="23" t="n">
+        <f aca="false">AVERAGE(E3:E7)</f>
+        <v>30.354</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <f aca="false">AVERAGE(F3:F7)</f>
+        <v>0.5636</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <f aca="false">STDEV(D3:D7)</f>
+        <v>0.0219818106624545</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <f aca="false">STDEV(E3:E7)</f>
+        <v>1.50573237994007</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <f aca="false">STDEV(F3:F7)</f>
+        <v>0.0265857104475317</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -6399,6 +7095,159 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>365414</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="17" t="n">
+        <v>-3.547</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>44.85</v>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>0.237</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>131053</v>
+      </c>
+      <c r="C4" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>-4.138</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>75.89</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>0.049</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>122026</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>-0.613</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>31.58</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>0.048</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>105108</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="19"/>
+      <c r="E6" s="9" t="n">
+        <v>49.81</v>
+      </c>
+      <c r="F6" s="19"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <f aca="false">AVERAGE(D3:D6)</f>
+        <v>-2.766</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <f aca="false">AVERAGE(E3:E6)</f>
+        <v>50.5325</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <f aca="false">AVERAGE(F3:F6)</f>
+        <v>0.111333333333333</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6418,38 +7267,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>60</v>
@@ -6471,7 +7320,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>61</v>
@@ -6493,7 +7342,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>62</v>
@@ -6515,7 +7364,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>63</v>
@@ -6537,7 +7386,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>60</v>
@@ -6563,7 +7412,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>61</v>
@@ -6589,7 +7438,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>62</v>
@@ -6615,7 +7464,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>63</v>
@@ -6637,7 +7486,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>60</v>
@@ -6663,7 +7512,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>61</v>
@@ -6689,7 +7538,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>62</v>
@@ -6715,7 +7564,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>63</v>
@@ -6737,7 +7586,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>60</v>
@@ -6763,7 +7612,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>61</v>
@@ -6789,7 +7638,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>62</v>
@@ -6815,7 +7664,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>63</v>
@@ -6837,29 +7686,29 @@
     </row>
     <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="C21" s="2" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B22" s="14" t="n">
         <f aca="false">AVERAGEIF($A$3:$A$18,$A22,E$3:E$18)</f>
@@ -6874,7 +7723,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B23" s="15" t="n">
         <f aca="false">AVERAGEIF($A$3:$A$18,$A23,E$3:E$18)</f>
@@ -6895,7 +7744,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B24" s="14" t="n">
         <f aca="false">AVERAGEIF($A$3:$A$18,$A24,E$3:E$18)</f>
@@ -6916,7 +7765,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="B25" s="15" t="n">
         <f aca="false">AVERAGEIF($A$3:$A$18,$A25,E$3:E$18)</f>
@@ -6937,39 +7786,39 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6977,13 +7826,13 @@
         <v>60</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>41</v>
@@ -6994,16 +7843,16 @@
         <v>61</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7011,16 +7860,16 @@
         <v>62</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7028,166 +7877,16 @@
         <v>63</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>41</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="23" t="n">
-        <v>0.2225</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="24" t="n">
-        <v>0.1306</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="23" t="n">
-        <v>0.0494</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>0.0427</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B7" s="23" t="n">
-        <v>0.0409</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B8" s="24" t="n">
-        <v>0.0156</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="23" t="n">
-        <v>0.0094</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="B14" s="23" t="n">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="B15" s="24" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B16" s="23" t="n">
-        <v>0.323</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="B17" s="24" t="n">
-        <v>29.7</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B18" s="23" t="n">
-        <v>723601</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustes UCS referencial ~ PEP: roca intacta vs todo, por registro y agrupado por litologia; figura del mejor ajuste y hoja Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT9AkNnHr1e9AMWji6YncB
</commit_message>
<xml_diff>
--- a/figuras/finales/tablas_capitulo6.xlsx
+++ b/figuras/finales/tablas_capitulo6.xlsx
@@ -22,10 +22,11 @@
     <sheet name="Comparación" sheetId="12" state="visible" r:id="rId14"/>
     <sheet name="UCS por litología" sheetId="13" state="visible" r:id="rId15"/>
     <sheet name="PEP estratos" sheetId="14" state="visible" r:id="rId16"/>
-    <sheet name="Concordancia 1541" sheetId="15" state="visible" r:id="rId17"/>
-    <sheet name="T6.3 Dominios" sheetId="16" state="visible" r:id="rId18"/>
-    <sheet name="T6.4 Ranking" sheetId="17" state="visible" r:id="rId19"/>
-    <sheet name="Bloques" sheetId="18" state="visible" r:id="rId20"/>
+    <sheet name="PEP ajustes" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="Concordancia 1541" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="T6.3 Dominios" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="T6.4 Ranking" sheetId="18" state="visible" r:id="rId20"/>
+    <sheet name="Bloques" sheetId="19" state="visible" r:id="rId21"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="391">
   <si>
     <t xml:space="preserve">Configuración de la corrida final (2026-10-22)</t>
   </si>
@@ -852,6 +853,120 @@
     <t xml:space="preserve">717.526 registros entrenables de roca intacta con PEP ≤ 1000 y ROP ≥ 0.2 m/min; 506 excluidos por PEP &gt; 1000 (ROP ≈ 0).</t>
   </si>
   <si>
+    <t xml:space="preserve">Ajustes UCS referencial ~ PEP: conjunto, agregación y forma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conjunto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agregación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puntos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² lineal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² parabólico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² potencial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² exponencial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² logarítmico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo roca intacta (DI ≤ 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por registro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por litología</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Litología × caserón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Litología × estrato de PP (10 bar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todo (intacta + fracturada)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² medido en MPa para todas las formas. Con 4 grupos la parábola tiene un solo grado de libertad: su R² no es comparable con el de 55 o 717.526 puntos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ecuaciones del ajuste parabólico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ecuación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo roca intacta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.00030255·PEP² + 0.32726·PEP + 77.217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.016577·PEP² + 12.826·PEP + -2296.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.012783·PEP² + 9.9608·PEP + -1762.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.0015059·PEP² + 1.2786·PEP + -132.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.00030452·PEP² + 0.33871·PEP + 71.851</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.014875·PEP² + 11.483·PEP + -2033.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.011707·PEP² + 9.1163·PEP + -1597.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCS = -0.002051·PEP² + 1.6513·PEP + -192.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grupos litología × caserón (conjunto todo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grupo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bht · PCC_0042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bht · PCC_1541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bht · PCS_1043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brecha_mixta · PCS_1043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kpcli · PCC_0042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kpcli · PCS_1043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kpcli · PCS_1059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kpcls · PCC_1541</t>
+  </si>
+  <si>
     <t xml:space="preserve">Picos de DI y cruces de malla en PCC_1541 (radio 3 m)</t>
   </si>
   <si>
@@ -886,9 +1001,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tabla 6.3 · Agrupación de dominios geomecánicos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grupo</t>
   </si>
   <si>
     <t xml:space="preserve">Estructura</t>
@@ -4359,6 +4471,597 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>717526</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>717526</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="G3" s="22" t="n">
+        <v>0.0407</v>
+      </c>
+      <c r="H3" s="22" t="n">
+        <v>0.0591</v>
+      </c>
+      <c r="I3" s="22" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="J3" s="22" t="n">
+        <v>0.0101</v>
+      </c>
+      <c r="K3" s="22" t="n">
+        <v>0.0518</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>717526</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="G4" s="23" t="n">
+        <v>0.0823</v>
+      </c>
+      <c r="H4" s="23" t="n">
+        <v>0.9888</v>
+      </c>
+      <c r="I4" s="23" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="J4" s="23" t="n">
+        <v>-0.0098</v>
+      </c>
+      <c r="K4" s="23" t="n">
+        <v>0.118</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>717526</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0.1635</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>0.7115</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>0.1126</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.0836</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <v>0.2013</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>717525</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>0.0635</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>0.1989</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>0.0261</v>
+      </c>
+      <c r="J6" s="23" t="n">
+        <v>-0.0094</v>
+      </c>
+      <c r="K6" s="23" t="n">
+        <v>0.0944</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>857980</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>857980</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>0.228</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="G7" s="22" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <v>0.0686</v>
+      </c>
+      <c r="I7" s="22" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="J7" s="22" t="n">
+        <v>0.0139</v>
+      </c>
+      <c r="K7" s="22" t="n">
+        <v>0.0613</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>857980</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>0.299</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>0.0896</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>0.9854</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>0.0177</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <v>-0.0058</v>
+      </c>
+      <c r="K8" s="23" t="n">
+        <v>0.1292</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>857980</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>0.417</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>0.1736</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>0.7211</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>0.1208</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.0892</v>
+      </c>
+      <c r="K9" s="22" t="n">
+        <v>0.2148</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>857978</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>0.2246</v>
+      </c>
+      <c r="I10" s="23" t="n">
+        <v>0.0282</v>
+      </c>
+      <c r="J10" s="23" t="n">
+        <v>-0.0046</v>
+      </c>
+      <c r="K10" s="23" t="n">
+        <v>0.0963</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>0.0591</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="D16" s="23" t="n">
+        <v>0.9888</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>0.7115</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D18" s="23" t="n">
+        <v>0.1989</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <v>0.0686</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>0.9854</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="D21" s="22" t="n">
+        <v>0.7211</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="D22" s="23" t="n">
+        <v>0.2246</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>335</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>128.1</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>307.8</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>128.1</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>352.7</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>128.1</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>454.7</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>111.5</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>352.8</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>431.7</v>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>376.4</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="B33" s="15" t="n">
+        <v>294.2</v>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4373,30 +5076,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>271</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>272</v>
+        <v>310</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>96</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>273</v>
+        <v>311</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>274</v>
+        <v>312</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>275</v>
+        <v>313</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>276</v>
+        <v>314</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>277</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4593,15 +5296,15 @@
     </row>
     <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>278</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>279</v>
+        <v>317</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>280</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4622,7 +5325,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="35" t="s">
-        <v>281</v>
+        <v>319</v>
       </c>
       <c r="B16" s="36" t="n">
         <v>0.152</v>
@@ -4647,7 +5350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4665,41 +5368,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>282</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>284</v>
+        <v>321</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>285</v>
+        <v>322</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>125</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>286</v>
+        <v>323</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>287</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>288</v>
+        <v>325</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>289</v>
+        <v>326</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>164.932209858122</v>
@@ -4716,13 +5419,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>291</v>
+        <v>328</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D4" s="15" t="n">
         <v>138.496561143358</v>
@@ -4739,13 +5442,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>293</v>
+        <v>330</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>294</v>
+        <v>331</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>134.789098647061</v>
@@ -4762,13 +5465,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>295</v>
+        <v>332</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>289</v>
+        <v>326</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>154.123768904038</v>
@@ -4785,13 +5488,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>296</v>
+        <v>333</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>289</v>
+        <v>326</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>137.155726282</v>
@@ -4808,13 +5511,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>297</v>
+        <v>334</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>298</v>
+        <v>335</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>139.393544557154</v>
@@ -4831,13 +5534,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>299</v>
+        <v>336</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>300</v>
+        <v>337</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>153.727676276695</v>
@@ -4854,13 +5557,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>301</v>
+        <v>338</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>168.41475157952</v>
@@ -4877,13 +5580,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>302</v>
+        <v>339</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>144.172700603197</v>
@@ -4900,13 +5603,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>303</v>
+        <v>340</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>304</v>
+        <v>341</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>159.684160752595</v>
@@ -4923,13 +5626,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>305</v>
+        <v>342</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>289</v>
+        <v>326</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>304</v>
+        <v>341</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>167.800529418651</v>
@@ -4946,13 +5649,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>306</v>
+        <v>343</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>294</v>
+        <v>331</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>298</v>
+        <v>335</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>124.601455398543</v>
@@ -4969,13 +5672,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>307</v>
+        <v>344</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>119.768508894793</v>
@@ -4992,13 +5695,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>308</v>
+        <v>345</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>294</v>
+        <v>331</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>119.704137883813</v>
@@ -5015,13 +5718,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>309</v>
+        <v>346</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>294</v>
+        <v>331</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>158.678228976082</v>
@@ -5038,7 +5741,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>310</v>
+        <v>347</v>
       </c>
     </row>
   </sheetData>
@@ -5052,7 +5755,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -5072,45 +5775,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>311</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>312</v>
+        <v>349</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>313</v>
+        <v>350</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>314</v>
+        <v>351</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>315</v>
+        <v>352</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>316</v>
+        <v>353</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>317</v>
+        <v>354</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>318</v>
+        <v>355</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>319</v>
+        <v>356</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>320</v>
+        <v>357</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>250</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>321</v>
+        <v>358</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>322</v>
+        <v>359</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>34</v>
@@ -5118,7 +5821,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>323</v>
+        <v>360</v>
       </c>
       <c r="B3" s="16" t="n">
         <v>1</v>
@@ -5148,7 +5851,7 @@
         <v>0.0048</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>324</v>
+        <v>361</v>
       </c>
       <c r="L3" s="14" t="n">
         <v>18.033</v>
@@ -5159,7 +5862,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>323</v>
+        <v>360</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>2</v>
@@ -5189,7 +5892,7 @@
         <v>0.0095</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>325</v>
+        <v>362</v>
       </c>
       <c r="L4" s="15" t="n">
         <v>23.376</v>
@@ -5200,7 +5903,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>323</v>
+        <v>360</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>3</v>
@@ -5230,7 +5933,7 @@
         <v>0.0117</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>326</v>
+        <v>363</v>
       </c>
       <c r="L5" s="14" t="n">
         <v>10.993</v>
@@ -5241,7 +5944,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>323</v>
+        <v>360</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>4</v>
@@ -5271,7 +5974,7 @@
         <v>0.0128</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>327</v>
+        <v>364</v>
       </c>
       <c r="L6" s="15" t="n">
         <v>28.854</v>
@@ -5282,7 +5985,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>323</v>
+        <v>360</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>5</v>
@@ -5312,7 +6015,7 @@
         <v>0.0172</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>328</v>
+        <v>365</v>
       </c>
       <c r="L7" s="14" t="n">
         <v>17.351</v>
@@ -5323,7 +6026,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>329</v>
+        <v>366</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>1</v>
@@ -5353,7 +6056,7 @@
         <v>0.1651</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>330</v>
+        <v>367</v>
       </c>
       <c r="L8" s="15" t="n">
         <v>20.324</v>
@@ -5364,7 +6067,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>329</v>
+        <v>366</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>2</v>
@@ -5405,7 +6108,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>329</v>
+        <v>366</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>3</v>
@@ -5435,7 +6138,7 @@
         <v>0.0715</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>331</v>
+        <v>368</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>19.494</v>
@@ -5446,7 +6149,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>329</v>
+        <v>366</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>4</v>
@@ -5476,7 +6179,7 @@
         <v>0.0977</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>331</v>
+        <v>368</v>
       </c>
       <c r="L11" s="14" t="n">
         <v>18.798</v>
@@ -5487,7 +6190,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>329</v>
+        <v>366</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>5</v>
@@ -5517,7 +6220,7 @@
         <v>0.1226</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>332</v>
+        <v>369</v>
       </c>
       <c r="L12" s="15" t="n">
         <v>20.774</v>
@@ -5528,7 +6231,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>333</v>
+        <v>370</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>1</v>
@@ -5558,7 +6261,7 @@
         <v>0.1226</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>332</v>
+        <v>369</v>
       </c>
       <c r="L13" s="14" t="n">
         <v>20.774</v>
@@ -5569,7 +6272,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>333</v>
+        <v>370</v>
       </c>
       <c r="B14" s="18" t="n">
         <v>2</v>
@@ -5599,7 +6302,7 @@
         <v>0.1651</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>330</v>
+        <v>367</v>
       </c>
       <c r="L14" s="15" t="n">
         <v>20.324</v>
@@ -5610,7 +6313,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>333</v>
+        <v>370</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>3</v>
@@ -5640,7 +6343,7 @@
         <v>0.1055</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>334</v>
+        <v>371</v>
       </c>
       <c r="L15" s="14" t="n">
         <v>28.608</v>
@@ -5651,7 +6354,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>333</v>
+        <v>370</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>4</v>
@@ -5681,7 +6384,7 @@
         <v>0.0952</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>335</v>
+        <v>372</v>
       </c>
       <c r="L16" s="15" t="n">
         <v>20.049</v>
@@ -5692,7 +6395,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>333</v>
+        <v>370</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>5</v>
@@ -5722,7 +6425,7 @@
         <v>0.0423</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>336</v>
+        <v>373</v>
       </c>
       <c r="L17" s="14" t="n">
         <v>28.47</v>
@@ -5742,7 +6445,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -5758,7 +6461,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>337</v>
+        <v>374</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5766,13 +6469,13 @@
         <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>338</v>
+        <v>375</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>287</v>
+        <v>324</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>339</v>
+        <v>376</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5846,7 +6549,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>279</v>
+        <v>317</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>2</v>
@@ -5854,7 +6557,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>340</v>
+        <v>377</v>
       </c>
       <c r="B10" s="24" t="n">
         <v>233015.6</v>
@@ -5862,7 +6565,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>341</v>
+        <v>378</v>
       </c>
       <c r="B11" s="21" t="n">
         <v>0.085</v>
@@ -5870,7 +6573,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>342</v>
+        <v>379</v>
       </c>
       <c r="B12" s="24" t="n">
         <v>0.73</v>
@@ -5878,7 +6581,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>343</v>
+        <v>380</v>
       </c>
       <c r="B13" s="25" t="n">
         <v>154.4</v>
@@ -5886,7 +6589,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>344</v>
+        <v>381</v>
       </c>
       <c r="B14" s="24" t="n">
         <v>130.9</v>
@@ -5894,7 +6597,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>345</v>
+        <v>382</v>
       </c>
       <c r="B15" s="25" t="n">
         <v>170.2</v>
@@ -5902,26 +6605,26 @@
     </row>
     <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>346</v>
+        <v>383</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>347</v>
+        <v>384</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>348</v>
+        <v>385</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>338</v>
+        <v>375</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>349</v>
+        <v>386</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>350</v>
+        <v>387</v>
       </c>
       <c r="C19" s="7" t="n">
         <v>1159</v>
@@ -5929,10 +6632,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>350</v>
+        <v>387</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>13651</v>
@@ -5940,10 +6643,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>352</v>
+        <v>389</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>350</v>
+        <v>387</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>103</v>
@@ -5951,7 +6654,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>353</v>
+        <v>390</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Desfase pico-cruce y sensibilidad al umbral para 4 caserones, PCC_0042 y PCC_1541: script, figura y hoja Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT9AkNnHr1e9AMWji6YncB
</commit_message>
<xml_diff>
--- a/figuras/finales/tablas_capitulo6.xlsx
+++ b/figuras/finales/tablas_capitulo6.xlsx
@@ -24,9 +24,10 @@
     <sheet name="PEP estratos" sheetId="14" state="visible" r:id="rId16"/>
     <sheet name="PEP ajustes" sheetId="15" state="visible" r:id="rId17"/>
     <sheet name="Concordancia 1541" sheetId="16" state="visible" r:id="rId18"/>
-    <sheet name="T6.3 Dominios" sheetId="17" state="visible" r:id="rId19"/>
-    <sheet name="T6.4 Ranking" sheetId="18" state="visible" r:id="rId20"/>
-    <sheet name="Bloques" sheetId="19" state="visible" r:id="rId21"/>
+    <sheet name="Concordancia caserones" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="T6.3 Dominios" sheetId="18" state="visible" r:id="rId20"/>
+    <sheet name="T6.4 Ranking" sheetId="19" state="visible" r:id="rId21"/>
+    <sheet name="Bloques" sheetId="20" state="visible" r:id="rId22"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="401">
   <si>
     <t xml:space="preserve">Configuración de la corrida final (2026-10-22)</t>
   </si>
@@ -998,6 +999,36 @@
   </si>
   <si>
     <t xml:space="preserve">Mediana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picos de DI y cruces de malla: 4 caserones, PCC_0042 (calibración) y PCC_1541 (prueba)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pozos con cruces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picos (umbral 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desfase medio [m]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desfase mediano [m]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">σ desfase [m]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensibilidad al umbral — 4 caserones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensibilidad al umbral — PCC_0042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensibilidad al umbral — PCC_1541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radio de concordancia 3 m; picos fusionados a &lt; 0,5 m; azar: mismos picos recolocados al azar en su pozo (30 repeticiones).</t>
   </si>
   <si>
     <t xml:space="preserve">Tabla 6.3 · Agrupación de dominios geomecánicos</t>
@@ -5355,6 +5386,794 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G40"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>928</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>450</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>4127</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>7.307</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>436</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>143</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>1527</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>-6.488</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>-4.235</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>8.62</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>237</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>187</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1320</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>-0.076</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>5.464</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>2463</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>0.439301664636622</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>0.668417104276069</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>0.439707673568819</v>
+      </c>
+      <c r="G9" s="31" t="n">
+        <f aca="false">D9-F9</f>
+        <v>-0.0004060089321965</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>3861</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>0.484071484071484</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0.874718679669918</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>0.450876284209618</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <f aca="false">D10-F10</f>
+        <v>0.0331951998618666</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>4127</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>0.50181730070269</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>0.924231057764441</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>0.4622970680882</v>
+      </c>
+      <c r="G11" s="31" t="n">
+        <f aca="false">D11-F11</f>
+        <v>0.03952023261449</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>3702</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>0.483792544570502</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0.880720180045011</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>0.465361066090402</v>
+      </c>
+      <c r="G12" s="32" t="n">
+        <f aca="false">D12-F12</f>
+        <v>0.0184314784801009</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>3109</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>0.486973303312962</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>0.807201800450113</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>0.460448161252278</v>
+      </c>
+      <c r="G13" s="31" t="n">
+        <f aca="false">D13-F13</f>
+        <v>0.026525142060684</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>2185</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>0.462700228832952</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>0.651162790697675</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>0.450511060259344</v>
+      </c>
+      <c r="G14" s="32" t="n">
+        <f aca="false">D14-F14</f>
+        <v>0.0121891685736078</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>0.44885993485342</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>0.516129032258065</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>0.447318132464712</v>
+      </c>
+      <c r="G15" s="31" t="n">
+        <f aca="false">D15-F15</f>
+        <v>0.00154180238870799</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>1016</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>1333</v>
+      </c>
+      <c r="D16" s="21" t="n">
+        <v>0.424212598425197</v>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>0.355588897224306</v>
+      </c>
+      <c r="F16" s="21" t="n">
+        <v>0.423950131233596</v>
+      </c>
+      <c r="G16" s="32" t="n">
+        <f aca="false">D16-F16</f>
+        <v>0.000262467191601057</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>1165</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>327</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>0.315021459227468</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>0.776758409785933</v>
+      </c>
+      <c r="F20" s="20" t="n">
+        <v>0.298226037195994</v>
+      </c>
+      <c r="G20" s="31" t="n">
+        <f aca="false">D20-F20</f>
+        <v>0.0167954220314736</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>1663</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>327</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>0.354780517137703</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>0.957186544342508</v>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0.314291441170575</v>
+      </c>
+      <c r="G21" s="32" t="n">
+        <f aca="false">D21-F21</f>
+        <v>0.0404890759671276</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>1527</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>327</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>0.366077275703995</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>0.960244648318043</v>
+      </c>
+      <c r="F22" s="20" t="n">
+        <v>0.310674525212836</v>
+      </c>
+      <c r="G22" s="31" t="n">
+        <f aca="false">D22-F22</f>
+        <v>0.0554027504911592</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>327</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>0.935779816513762</v>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>0.311666666666667</v>
+      </c>
+      <c r="G23" s="32" t="n">
+        <f aca="false">D23-F23</f>
+        <v>0.0633333333333334</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>1211</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>327</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>0.380677126341866</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>0.883792048929664</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>0.311202862647949</v>
+      </c>
+      <c r="G24" s="31" t="n">
+        <f aca="false">D24-F24</f>
+        <v>0.0694742636939168</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>930</v>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>327</v>
+      </c>
+      <c r="D25" s="21" t="n">
+        <v>0.348387096774194</v>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>0.755351681957187</v>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.320645161290323</v>
+      </c>
+      <c r="G25" s="32" t="n">
+        <f aca="false">D25-F25</f>
+        <v>0.0277419354838709</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>673</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>327</v>
+      </c>
+      <c r="D26" s="20" t="n">
+        <v>0.337295690936107</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>0.648318042813456</v>
+      </c>
+      <c r="F26" s="20" t="n">
+        <v>0.30975730559683</v>
+      </c>
+      <c r="G26" s="31" t="n">
+        <f aca="false">D26-F26</f>
+        <v>0.0275383853392768</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" s="10" t="n">
+        <v>481</v>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>327</v>
+      </c>
+      <c r="D27" s="21" t="n">
+        <v>0.355509355509356</v>
+      </c>
+      <c r="E27" s="21" t="n">
+        <v>0.501529051987768</v>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>0.299376299376299</v>
+      </c>
+      <c r="G27" s="32" t="n">
+        <f aca="false">D27-F27</f>
+        <v>0.0561330561330561</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>297</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>0.521885521885522</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>0.407228915662651</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>0.543097643097643</v>
+      </c>
+      <c r="G31" s="31" t="n">
+        <f aca="false">D31-F31</f>
+        <v>-0.0212121212121211</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>773</v>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D32" s="21" t="n">
+        <v>0.580853816300129</v>
+      </c>
+      <c r="E32" s="21" t="n">
+        <v>0.727710843373494</v>
+      </c>
+      <c r="F32" s="21" t="n">
+        <v>0.519879258300992</v>
+      </c>
+      <c r="G32" s="32" t="n">
+        <f aca="false">D32-F32</f>
+        <v>0.0609745579991374</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>1320</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>0.58030303030303</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>0.927710843373494</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <v>0.526414141414141</v>
+      </c>
+      <c r="G33" s="31" t="n">
+        <f aca="false">D33-F33</f>
+        <v>0.0538888888888889</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D34" s="21" t="n">
+        <v>0.514166666666667</v>
+      </c>
+      <c r="E34" s="21" t="n">
+        <v>0.857831325301205</v>
+      </c>
+      <c r="F34" s="21" t="n">
+        <v>0.525722222222222</v>
+      </c>
+      <c r="G34" s="32" t="n">
+        <f aca="false">D34-F34</f>
+        <v>-0.0115555555555555</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>893</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D35" s="20" t="n">
+        <v>0.516237402015678</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <v>0.734939759036145</v>
+      </c>
+      <c r="F35" s="20" t="n">
+        <v>0.522471071295259</v>
+      </c>
+      <c r="G35" s="31" t="n">
+        <f aca="false">D35-F35</f>
+        <v>-0.00623366927958191</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>505</v>
+      </c>
+      <c r="C36" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D36" s="21" t="n">
+        <v>0.524752475247525</v>
+      </c>
+      <c r="E36" s="21" t="n">
+        <v>0.563855421686747</v>
+      </c>
+      <c r="F36" s="21" t="n">
+        <v>0.52019801980198</v>
+      </c>
+      <c r="G36" s="32" t="n">
+        <f aca="false">D36-F36</f>
+        <v>0.00455445544554456</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>316</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D37" s="20" t="n">
+        <v>0.541139240506329</v>
+      </c>
+      <c r="E37" s="20" t="n">
+        <v>0.414457831325301</v>
+      </c>
+      <c r="F37" s="20" t="n">
+        <v>0.517405063291139</v>
+      </c>
+      <c r="G37" s="31" t="n">
+        <f aca="false">D37-F37</f>
+        <v>0.02373417721519</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B38" s="10" t="n">
+        <v>178</v>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D38" s="21" t="n">
+        <v>0.443820224719101</v>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>0.214457831325301</v>
+      </c>
+      <c r="F38" s="21" t="n">
+        <v>0.498689138576779</v>
+      </c>
+      <c r="G38" s="32" t="n">
+        <f aca="false">D38-F38</f>
+        <v>-0.0548689138576779</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
+        <v>329</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5368,7 +6187,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5379,30 +6198,30 @@
         <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>125</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>164.932209858122</v>
@@ -5419,13 +6238,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D4" s="15" t="n">
         <v>138.496561143358</v>
@@ -5442,13 +6261,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>134.789098647061</v>
@@ -5465,13 +6284,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>154.123768904038</v>
@@ -5488,13 +6307,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>137.155726282</v>
@@ -5511,13 +6330,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>139.393544557154</v>
@@ -5534,13 +6353,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>337</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>327</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>153.727676276695</v>
@@ -5557,13 +6376,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>168.41475157952</v>
@@ -5580,13 +6399,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>329</v>
-      </c>
       <c r="C11" s="3" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>144.172700603197</v>
@@ -5603,13 +6422,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>159.684160752595</v>
@@ -5626,13 +6445,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>167.800529418651</v>
@@ -5649,13 +6468,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>124.601455398543</v>
@@ -5672,13 +6491,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>344</v>
+        <v>354</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>119.768508894793</v>
@@ -5695,13 +6514,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>345</v>
+        <v>355</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>119.704137883813</v>
@@ -5718,13 +6537,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>158.678228976082</v>
@@ -5741,7 +6560,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>347</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>
@@ -5755,7 +6574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -5775,45 +6594,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>250</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>34</v>
@@ -5821,7 +6640,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="B3" s="16" t="n">
         <v>1</v>
@@ -5851,7 +6670,7 @@
         <v>0.0048</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="L3" s="14" t="n">
         <v>18.033</v>
@@ -5862,7 +6681,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>2</v>
@@ -5892,7 +6711,7 @@
         <v>0.0095</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
       <c r="L4" s="15" t="n">
         <v>23.376</v>
@@ -5903,7 +6722,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>3</v>
@@ -5933,7 +6752,7 @@
         <v>0.0117</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
       <c r="L5" s="14" t="n">
         <v>10.993</v>
@@ -5944,7 +6763,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>4</v>
@@ -5974,7 +6793,7 @@
         <v>0.0128</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="L6" s="15" t="n">
         <v>28.854</v>
@@ -5985,7 +6804,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>5</v>
@@ -6015,7 +6834,7 @@
         <v>0.0172</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="L7" s="14" t="n">
         <v>17.351</v>
@@ -6026,7 +6845,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>1</v>
@@ -6056,7 +6875,7 @@
         <v>0.1651</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
       <c r="L8" s="15" t="n">
         <v>20.324</v>
@@ -6067,7 +6886,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>2</v>
@@ -6108,7 +6927,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>3</v>
@@ -6138,7 +6957,7 @@
         <v>0.0715</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>19.494</v>
@@ -6149,7 +6968,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>4</v>
@@ -6179,7 +6998,7 @@
         <v>0.0977</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="L11" s="14" t="n">
         <v>18.798</v>
@@ -6190,7 +7009,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>5</v>
@@ -6220,7 +7039,7 @@
         <v>0.1226</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="L12" s="15" t="n">
         <v>20.774</v>
@@ -6231,7 +7050,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>1</v>
@@ -6261,7 +7080,7 @@
         <v>0.1226</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="L13" s="14" t="n">
         <v>20.774</v>
@@ -6272,7 +7091,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="B14" s="18" t="n">
         <v>2</v>
@@ -6302,7 +7121,7 @@
         <v>0.1651</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
       <c r="L14" s="15" t="n">
         <v>20.324</v>
@@ -6313,7 +7132,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>3</v>
@@ -6343,7 +7162,7 @@
         <v>0.1055</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
       <c r="L15" s="14" t="n">
         <v>28.608</v>
@@ -6354,7 +7173,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>4</v>
@@ -6384,7 +7203,7 @@
         <v>0.0952</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="L16" s="15" t="n">
         <v>20.049</v>
@@ -6395,7 +7214,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>5</v>
@@ -6425,236 +7244,13 @@
         <v>0.0423</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="L17" s="14" t="n">
         <v>28.47</v>
       </c>
       <c r="M17" s="16" t="n">
         <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" s="7" t="n">
-        <v>6729</v>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>424184</v>
-      </c>
-      <c r="D3" s="20" t="n">
-        <v>0.3172</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="10" t="n">
-        <v>3244</v>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>176898</v>
-      </c>
-      <c r="D4" s="21" t="n">
-        <v>0.2555</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>3356</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>141577</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>0.233</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>1584</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>126768</v>
-      </c>
-      <c r="D6" s="21" t="n">
-        <v>0.2266</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="5" t="n">
-        <f aca="false">SUM(B3:B6)</f>
-        <v>14913</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <f aca="false">SUM(C3:C6)</f>
-        <v>869427</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="B10" s="24" t="n">
-        <v>233015.6</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>0.085</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="B12" s="24" t="n">
-        <v>0.73</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>380</v>
-      </c>
-      <c r="B13" s="25" t="n">
-        <v>154.4</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="B14" s="24" t="n">
-        <v>130.9</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>382</v>
-      </c>
-      <c r="B15" s="25" t="n">
-        <v>170.2</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>1159</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>388</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>387</v>
-      </c>
-      <c r="C20" s="10" t="n">
-        <v>13651</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -6864,6 +7460,229 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
         <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>6729</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>424184</v>
+      </c>
+      <c r="D3" s="20" t="n">
+        <v>0.3172</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>3244</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>176898</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>0.2555</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>3356</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>141577</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>0.233</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>1584</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>126768</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>0.2266</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <f aca="false">SUM(B3:B6)</f>
+        <v>14913</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <f aca="false">SUM(C3:C6)</f>
+        <v>869427</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>233015.6</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>0.085</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="B13" s="25" t="n">
+        <v>154.4</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>130.9</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="B15" s="25" t="n">
+        <v>170.2</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>13651</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Matriz DI x UCS de bloques tambien en m3 (figura y hoja Excel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT9AkNnHr1e9AMWji6YncB
</commit_message>
<xml_diff>
--- a/figuras/finales/tablas_capitulo6.xlsx
+++ b/figuras/finales/tablas_capitulo6.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="408">
   <si>
     <t xml:space="preserve">Configuración de la corrida final (2026-10-22)</t>
   </si>
@@ -1220,25 +1220,46 @@
     <t xml:space="preserve">UCS P90 [MPa]</t>
   </si>
   <si>
+    <t xml:space="preserve">Clasificación DI × UCS de matriz — bloques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clase de DI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 125 MPa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">125–150 MPa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150–175 MPa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 175 MPa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sana (DI ≤ 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transición (1 &lt; DI ≤ 1,5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fracturada (DI &gt; 1,5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clasificación DI × UCS de matriz — volumen [m³]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloque de 2,5 m = 15.625 m³. Clases de UCS cada 25 MPa: todos los bloques caen en la banda ISRM R5.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bloques por clase de DI</t>
   </si>
   <si>
-    <t xml:space="preserve">Clase de DI</t>
-  </si>
-  <si>
     <t xml:space="preserve">Banda ISRM de UCS</t>
   </si>
   <si>
-    <t xml:space="preserve">transición (1 &lt; DI ≤ 1,5)</t>
-  </si>
-  <si>
     <t xml:space="preserve">R5 muy alta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sana (DI ≤ 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fracturada (DI &gt; 1,5)</t>
   </si>
   <si>
     <t xml:space="preserve">Aproximación de apoyo a la tronadura, no modelo geológico validado. Un bloque sin soporte de datos no se incluye.</t>
@@ -7478,13 +7499,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7644,45 +7666,276 @@
         <v>395</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>385</v>
+        <v>396</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>397</v>
+        <v>399</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>594</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>1159</v>
+        <v>4778</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>7925</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>354</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <f aca="false">SUM(B19:E19)</f>
+        <v>13651</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>397</v>
+        <v>400</v>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>19</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>13651</v>
+        <v>487</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>640</v>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <f aca="false">SUM(B20:E20)</f>
+        <v>1159</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <f aca="false">SUM(B21:E21)</f>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <f aca="false">SUM(B19:B21)</f>
+        <v>614</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <f aca="false">SUM(C19:C21)</f>
+        <v>5299</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <f aca="false">SUM(D19:D21)</f>
+        <v>8628</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <f aca="false">SUM(E19:E21)</f>
+        <v>372</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <f aca="false">SUM(F19:F21)</f>
+        <v>14913</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="C21" s="7" t="n">
+      <c r="B26" s="7" t="n">
+        <v>9281.25</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>74656.25</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>123828.125</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>5531.25</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <f aca="false">SUM(B26:E26)</f>
+        <v>213296.875</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="B27" s="10" t="n">
+        <v>296.875</v>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>7609.375</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>203.125</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <f aca="false">SUM(B27:E27)</f>
+        <v>18109.375</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>15.625</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>531.25</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>984.375</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>78.125</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <f aca="false">SUM(B28:E28)</f>
+        <v>1609.375</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <f aca="false">SUM(B26:B28)</f>
+        <v>9593.75</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <f aca="false">SUM(C26:C28)</f>
+        <v>82796.875</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <f aca="false">SUM(D26:D28)</f>
+        <v>134812.5</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <f aca="false">SUM(E26:E28)</f>
+        <v>5812.5</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <f aca="false">SUM(F26:F28)</f>
+        <v>233015.625</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>13651</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C36" s="7" t="n">
         <v>103</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>400</v>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ROP frente a PP, AP, RP y DP: correlacion simple, parcial e intra-pozo por litologia (figura y hoja Excel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT9AkNnHr1e9AMWji6YncB
</commit_message>
<xml_diff>
--- a/figuras/finales/tablas_capitulo6.xlsx
+++ b/figuras/finales/tablas_capitulo6.xlsx
@@ -23,11 +23,12 @@
     <sheet name="UCS por litología" sheetId="13" state="visible" r:id="rId15"/>
     <sheet name="PEP estratos" sheetId="14" state="visible" r:id="rId16"/>
     <sheet name="PEP ajustes" sheetId="15" state="visible" r:id="rId17"/>
-    <sheet name="Concordancia 1541" sheetId="16" state="visible" r:id="rId18"/>
-    <sheet name="Concordancia caserones" sheetId="17" state="visible" r:id="rId19"/>
-    <sheet name="T6.3 Dominios" sheetId="18" state="visible" r:id="rId20"/>
-    <sheet name="T6.4 Ranking" sheetId="19" state="visible" r:id="rId21"/>
-    <sheet name="Bloques" sheetId="20" state="visible" r:id="rId22"/>
+    <sheet name="ROP vs presiones" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="Concordancia 1541" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="Concordancia caserones" sheetId="18" state="visible" r:id="rId20"/>
+    <sheet name="T6.3 Dominios" sheetId="19" state="visible" r:id="rId21"/>
+    <sheet name="T6.4 Ranking" sheetId="20" state="visible" r:id="rId22"/>
+    <sheet name="Bloques" sheetId="21" state="visible" r:id="rId23"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="426">
   <si>
     <t xml:space="preserve">Configuración de la corrida final (2026-10-22)</t>
   </si>
@@ -966,6 +967,60 @@
   </si>
   <si>
     <t xml:space="preserve">Kpcls · PCC_1541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relación de la ROP con PP, AP, RP y DP (roca continua entrenable; FP excluida por criterio físico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ρ simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ρ parcial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ρ dentro del pozo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² sola (rangos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² las 4 (rangos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mediana [bar]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todas las litologías</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ρ parcial: rangos descontando linealmente las otras tres presiones. ρ dentro del pozo: desviaciones respecto de la mediana de cada pozo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlación entre presiones (todas las litologías)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Par</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PP-AP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PP-RP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PP-DP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AP-RP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AP-DP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RP-DP</t>
   </si>
   <si>
     <t xml:space="preserve">Picos de DI y cruces de malla en PCC_1541 (radio 3 m)</t>
@@ -5114,16 +5169,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5133,262 +5188,740 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="C2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>315</v>
       </c>
+      <c r="J2" s="2" t="s">
+        <v>316</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B3" s="7" t="n">
-        <v>297</v>
+      <c r="A3" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>415</v>
-      </c>
-      <c r="D3" s="20" t="n">
-        <v>0.521885521885522</v>
-      </c>
-      <c r="E3" s="20" t="n">
-        <v>0.407228915662651</v>
-      </c>
-      <c r="F3" s="20" t="n">
-        <v>0.543097643097643</v>
-      </c>
-      <c r="G3" s="31" t="n">
-        <f aca="false">D3-F3</f>
-        <v>-0.0212121212121211</v>
+        <v>718032</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>900</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="G3" s="17" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="H3" s="22" t="n">
+        <v>0.0553</v>
+      </c>
+      <c r="I3" s="22" t="n">
+        <v>0.1001</v>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>218.4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="B4" s="10" t="n">
-        <v>773</v>
+      <c r="A4" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>77</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>415</v>
-      </c>
-      <c r="D4" s="21" t="n">
-        <v>0.580853816300129</v>
-      </c>
-      <c r="E4" s="21" t="n">
-        <v>0.727710843373494</v>
-      </c>
-      <c r="F4" s="21" t="n">
-        <v>0.519879258300992</v>
-      </c>
-      <c r="G4" s="32" t="n">
-        <f aca="false">D4-F4</f>
-        <v>0.0609745579991374</v>
+        <v>718032</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>900</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="H4" s="23" t="n">
+        <v>0.0112</v>
+      </c>
+      <c r="I4" s="23" t="n">
+        <v>0.1001</v>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>76.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>1320</v>
+      <c r="A5" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>74</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>415</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>0.58030303030303</v>
-      </c>
-      <c r="E5" s="20" t="n">
-        <v>0.927710843373494</v>
-      </c>
-      <c r="F5" s="20" t="n">
-        <v>0.526414141414141</v>
-      </c>
-      <c r="G5" s="31" t="n">
-        <f aca="false">D5-F5</f>
-        <v>0.0538888888888889</v>
+        <v>718032</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>900</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>-0.181</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>-0.174</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>0.0327</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>0.1001</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>46.8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>1200</v>
+      <c r="A6" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>415</v>
-      </c>
-      <c r="D6" s="21" t="n">
-        <v>0.514166666666667</v>
-      </c>
-      <c r="E6" s="21" t="n">
-        <v>0.857831325301205</v>
-      </c>
-      <c r="F6" s="21" t="n">
-        <v>0.525722222222222</v>
-      </c>
-      <c r="G6" s="32" t="n">
-        <f aca="false">D6-F6</f>
-        <v>-0.0115555555555555</v>
+        <v>718032</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>900</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>-0.044</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>-0.136</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>-0.057</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>0.1001</v>
+      </c>
+      <c r="J6" s="15" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>893</v>
+      <c r="A7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>415</v>
-      </c>
-      <c r="D7" s="20" t="n">
-        <v>0.516237402015678</v>
-      </c>
-      <c r="E7" s="20" t="n">
-        <v>0.734939759036145</v>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>0.522471071295259</v>
-      </c>
-      <c r="G7" s="31" t="n">
-        <f aca="false">D7-F7</f>
-        <v>-0.00623366927958191</v>
+        <v>52992</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>188</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <v>0.0117</v>
+      </c>
+      <c r="I7" s="22" t="n">
+        <v>0.0509</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>217.6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="10" t="n">
-        <v>505</v>
+      <c r="A8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>77</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>415</v>
-      </c>
-      <c r="D8" s="21" t="n">
-        <v>0.524752475247525</v>
-      </c>
-      <c r="E8" s="21" t="n">
-        <v>0.563855421686747</v>
-      </c>
-      <c r="F8" s="21" t="n">
-        <v>0.52019801980198</v>
-      </c>
-      <c r="G8" s="32" t="n">
-        <f aca="false">D8-F8</f>
-        <v>0.00455445544554456</v>
+        <v>52992</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>188</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>0.0157</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>0.0509</v>
+      </c>
+      <c r="J8" s="15" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>316</v>
+      <c r="A9" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>74</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>415</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>0.541139240506329</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>0.414457831325301</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>0.517405063291139</v>
-      </c>
-      <c r="G9" s="31" t="n">
-        <f aca="false">D9-F9</f>
-        <v>0.02373417721519</v>
+        <v>52992</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>188</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>-0.123</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>0.0509</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>45.4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>178</v>
+      <c r="A10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>415</v>
-      </c>
-      <c r="D10" s="21" t="n">
-        <v>0.443820224719101</v>
-      </c>
-      <c r="E10" s="21" t="n">
-        <v>0.214457831325301</v>
-      </c>
-      <c r="F10" s="21" t="n">
-        <v>0.498689138576779</v>
-      </c>
-      <c r="G10" s="32" t="n">
-        <f aca="false">D10-F10</f>
-        <v>-0.0548689138576779</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>316</v>
+        <v>52992</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>188</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>-0.119</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="I10" s="23" t="n">
+        <v>0.0509</v>
+      </c>
+      <c r="J10" s="15" t="n">
+        <v>99.9</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>16787</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.1407</v>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>0.2251</v>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>179.9</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>16787</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="H12" s="23" t="n">
+        <v>0.0235</v>
+      </c>
+      <c r="I12" s="23" t="n">
+        <v>0.2251</v>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>76.4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="B13" s="2" t="s">
+      <c r="A13" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>16787</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>-0.195</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>-0.307</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="H13" s="22" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>0.2251</v>
+      </c>
+      <c r="J13" s="14" t="n">
+        <v>56.7</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>16787</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="H14" s="23" t="n">
+        <v>0.0189</v>
+      </c>
+      <c r="I14" s="23" t="n">
+        <v>0.2251</v>
+      </c>
+      <c r="J14" s="15" t="n">
+        <v>104.3</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>224091</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>487</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>-0.084</v>
+      </c>
+      <c r="H15" s="22" t="n">
+        <v>0.0605</v>
+      </c>
+      <c r="I15" s="22" t="n">
+        <v>0.0984</v>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>216.6</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>224091</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>487</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="H16" s="23" t="n">
+        <v>0.0251</v>
+      </c>
+      <c r="I16" s="23" t="n">
+        <v>0.0984</v>
+      </c>
+      <c r="J16" s="15" t="n">
+        <v>76.2</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>224091</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>487</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>-0.068</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>-0.066</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>-0.089</v>
+      </c>
+      <c r="H17" s="22" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="I17" s="22" t="n">
+        <v>0.0984</v>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>224091</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>487</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>-0.181</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>-0.068</v>
+      </c>
+      <c r="H18" s="23" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="I18" s="23" t="n">
+        <v>0.0984</v>
+      </c>
+      <c r="J18" s="15" t="n">
+        <v>101.8</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>424162</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>571</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="G19" s="17" t="n">
+        <v>-0.126</v>
+      </c>
+      <c r="H19" s="22" t="n">
+        <v>0.0435</v>
+      </c>
+      <c r="I19" s="22" t="n">
+        <v>0.0681</v>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>424162</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>571</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>0.084</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="H20" s="23" t="n">
+        <v>0.0109</v>
+      </c>
+      <c r="I20" s="23" t="n">
+        <v>0.0681</v>
+      </c>
+      <c r="J20" s="15" t="n">
+        <v>76.9</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>424162</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>571</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <v>-0.139</v>
+      </c>
+      <c r="F21" s="17" t="n">
+        <v>-0.117</v>
+      </c>
+      <c r="G21" s="17" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="H21" s="22" t="n">
+        <v>0.0193</v>
+      </c>
+      <c r="I21" s="22" t="n">
+        <v>0.0681</v>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>48.6</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>424162</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>571</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="H22" s="23" t="n">
+        <v>0.0006</v>
+      </c>
+      <c r="I22" s="23" t="n">
+        <v>0.0681</v>
+      </c>
+      <c r="J22" s="15" t="n">
+        <v>102.5</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>1320</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="33" t="s">
-        <v>175</v>
-      </c>
-      <c r="B15" s="34" t="n">
-        <v>-0.0758083333333332</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="35" t="s">
+    <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="B16" s="36" t="n">
-        <v>0.152</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="B17" s="9" t="n">
-        <v>5.46420883724733</v>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="B27" s="17" t="n">
+        <v>0.379</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="B28" s="19" t="n">
+        <v>-0.066</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B29" s="17" t="n">
+        <v>0.229</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>0.006</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>-0.008</v>
       </c>
     </row>
   </sheetData>
@@ -5407,6 +5940,299 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>297</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D3" s="20" t="n">
+        <v>0.521885521885522</v>
+      </c>
+      <c r="E3" s="20" t="n">
+        <v>0.407228915662651</v>
+      </c>
+      <c r="F3" s="20" t="n">
+        <v>0.543097643097643</v>
+      </c>
+      <c r="G3" s="31" t="n">
+        <f aca="false">D3-F3</f>
+        <v>-0.0212121212121211</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>773</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>0.580853816300129</v>
+      </c>
+      <c r="E4" s="21" t="n">
+        <v>0.727710843373494</v>
+      </c>
+      <c r="F4" s="21" t="n">
+        <v>0.519879258300992</v>
+      </c>
+      <c r="G4" s="32" t="n">
+        <f aca="false">D4-F4</f>
+        <v>0.0609745579991374</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1320</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>0.58030303030303</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>0.927710843373494</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>0.526414141414141</v>
+      </c>
+      <c r="G5" s="31" t="n">
+        <f aca="false">D5-F5</f>
+        <v>0.0538888888888889</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>0.514166666666667</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>0.857831325301205</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>0.525722222222222</v>
+      </c>
+      <c r="G6" s="32" t="n">
+        <f aca="false">D6-F6</f>
+        <v>-0.0115555555555555</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>893</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>0.516237402015678</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>0.734939759036145</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>0.522471071295259</v>
+      </c>
+      <c r="G7" s="31" t="n">
+        <f aca="false">D7-F7</f>
+        <v>-0.00623366927958191</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>505</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>0.524752475247525</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>0.563855421686747</v>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>0.52019801980198</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <f aca="false">D8-F8</f>
+        <v>0.00455445544554456</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>316</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>415</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>0.541139240506329</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>0.414457831325301</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>0.517405063291139</v>
+      </c>
+      <c r="G9" s="31" t="n">
+        <f aca="false">D9-F9</f>
+        <v>0.02373417721519</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>178</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>415</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>0.443820224719101</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0.214457831325301</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>0.498689138576779</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <f aca="false">D10-F10</f>
+        <v>-0.0548689138576779</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="33" t="s">
+        <v>175</v>
+      </c>
+      <c r="B15" s="34" t="n">
+        <v>-0.0758083333333332</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="35" t="s">
+        <v>337</v>
+      </c>
+      <c r="B16" s="36" t="n">
+        <v>0.152</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>5.46420883724733</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5419,7 +6245,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5430,19 +6256,19 @@
         <v>59</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>322</v>
+        <v>340</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>323</v>
+        <v>341</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>324</v>
+        <v>342</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5516,30 +6342,30 @@
     </row>
     <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>326</v>
+        <v>344</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>96</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5736,30 +6562,30 @@
     </row>
     <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>96</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5956,30 +6782,30 @@
     </row>
     <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>96</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6176,7 +7002,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
     </row>
   </sheetData>
@@ -6190,7 +7016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6208,7 +7034,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6219,30 +7045,30 @@
         <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>125</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>164.932209858122</v>
@@ -6259,13 +7085,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D4" s="15" t="n">
         <v>138.496561143358</v>
@@ -6282,13 +7108,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>134.789098647061</v>
@@ -6305,13 +7131,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>154.123768904038</v>
@@ -6328,13 +7154,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>137.155726282</v>
@@ -6351,13 +7177,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>139.393544557154</v>
@@ -6374,13 +7200,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>153.727676276695</v>
@@ -6397,13 +7223,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>168.41475157952</v>
@@ -6420,13 +7246,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>144.172700603197</v>
@@ -6443,13 +7269,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>159.684160752595</v>
@@ -6466,13 +7292,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>167.800529418651</v>
@@ -6489,13 +7315,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>353</v>
+        <v>371</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>124.601455398543</v>
@@ -6512,13 +7338,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>354</v>
+        <v>372</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>119.768508894793</v>
@@ -6535,13 +7361,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>355</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>337</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>119.704137883813</v>
@@ -6558,13 +7384,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>158.678228976082</v>
@@ -6581,697 +7407,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>357</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>365</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="B3" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="16" t="n">
-        <v>224.873875</v>
-      </c>
-      <c r="D3" s="16" t="n">
-        <v>51.426875</v>
-      </c>
-      <c r="E3" s="16" t="n">
-        <v>79.514375</v>
-      </c>
-      <c r="F3" s="16" t="n">
-        <v>110.959</v>
-      </c>
-      <c r="G3" s="14" t="n">
-        <v>8.208875</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>0.710875</v>
-      </c>
-      <c r="I3" s="16" t="n">
-        <v>500.540267735832</v>
-      </c>
-      <c r="J3" s="22" t="n">
-        <v>0.0048</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="L3" s="14" t="n">
-        <v>18.033</v>
-      </c>
-      <c r="M3" s="16" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="B4" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="18" t="n">
-        <v>224.9996</v>
-      </c>
-      <c r="D4" s="18" t="n">
-        <v>59.8344</v>
-      </c>
-      <c r="E4" s="18" t="n">
-        <v>85.172</v>
-      </c>
-      <c r="F4" s="18" t="n">
-        <v>118.3634</v>
-      </c>
-      <c r="G4" s="15" t="n">
-        <v>7.3848</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>0.9916</v>
-      </c>
-      <c r="I4" s="18" t="n">
-        <v>373.165042543947</v>
-      </c>
-      <c r="J4" s="23" t="n">
-        <v>0.0095</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="L4" s="15" t="n">
-        <v>23.376</v>
-      </c>
-      <c r="M4" s="18" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="B5" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>225.403142857143</v>
-      </c>
-      <c r="D5" s="16" t="n">
-        <v>50.718</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>74.8847142857143</v>
-      </c>
-      <c r="F5" s="16" t="n">
-        <v>102.72</v>
-      </c>
-      <c r="G5" s="14" t="n">
-        <v>8.483</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>0.872857142857143</v>
-      </c>
-      <c r="I5" s="16" t="n">
-        <v>402.175669000924</v>
-      </c>
-      <c r="J5" s="22" t="n">
-        <v>0.0117</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>373</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>10.993</v>
-      </c>
-      <c r="M5" s="16" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="B6" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="18" t="n">
-        <v>224.914</v>
-      </c>
-      <c r="D6" s="18" t="n">
-        <v>50.29</v>
-      </c>
-      <c r="E6" s="18" t="n">
-        <v>99.938</v>
-      </c>
-      <c r="F6" s="18" t="n">
-        <v>121.1454</v>
-      </c>
-      <c r="G6" s="15" t="n">
-        <v>7.5276</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>0.9376</v>
-      </c>
-      <c r="I6" s="18" t="n">
-        <v>400.204833233857</v>
-      </c>
-      <c r="J6" s="23" t="n">
-        <v>0.0128</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="L6" s="15" t="n">
-        <v>28.854</v>
-      </c>
-      <c r="M6" s="18" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="B7" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>223.309</v>
-      </c>
-      <c r="D7" s="16" t="n">
-        <v>42.6395</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>76.9009</v>
-      </c>
-      <c r="F7" s="16" t="n">
-        <v>110.745</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>9.1322</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>1.052</v>
-      </c>
-      <c r="I7" s="16" t="n">
-        <v>325.995300891542</v>
-      </c>
-      <c r="J7" s="22" t="n">
-        <v>0.0172</v>
-      </c>
-      <c r="K7" s="3" t="s">
         <v>375</v>
-      </c>
-      <c r="L7" s="14" t="n">
-        <v>17.351</v>
-      </c>
-      <c r="M7" s="16" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="B8" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="18" t="n">
-        <v>149.9926</v>
-      </c>
-      <c r="D8" s="18" t="n">
-        <v>52.8152</v>
-      </c>
-      <c r="E8" s="18" t="n">
-        <v>77.6606</v>
-      </c>
-      <c r="F8" s="18" t="n">
-        <v>75.8416</v>
-      </c>
-      <c r="G8" s="15" t="n">
-        <v>8.2484</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>1.787</v>
-      </c>
-      <c r="I8" s="18" t="n">
-        <v>162.332346613696</v>
-      </c>
-      <c r="J8" s="23" t="n">
-        <v>0.1651</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>377</v>
-      </c>
-      <c r="L8" s="15" t="n">
-        <v>20.324</v>
-      </c>
-      <c r="M8" s="18" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>376</v>
-      </c>
-      <c r="B9" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>119.5725</v>
-      </c>
-      <c r="D9" s="16" t="n">
-        <v>43.6025</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>52.6261666666667</v>
-      </c>
-      <c r="F9" s="16" t="n">
-        <v>56.389</v>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>8.07066666666667</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>1.36783333333333</v>
-      </c>
-      <c r="I9" s="16" t="n">
-        <v>166.827549144259</v>
-      </c>
-      <c r="J9" s="22" t="n">
-        <v>0.2719</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>26.594</v>
-      </c>
-      <c r="M9" s="16" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="B10" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="18" t="n">
-        <v>125.2542</v>
-      </c>
-      <c r="D10" s="18" t="n">
-        <v>39.7184</v>
-      </c>
-      <c r="E10" s="18" t="n">
-        <v>59.4492</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>73.224</v>
-      </c>
-      <c r="G10" s="15" t="n">
-        <v>9.3226</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>1.3474</v>
-      </c>
-      <c r="I10" s="18" t="n">
-        <v>167.32673415805</v>
-      </c>
-      <c r="J10" s="23" t="n">
-        <v>0.0715</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="L10" s="15" t="n">
-        <v>19.494</v>
-      </c>
-      <c r="M10" s="18" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>376</v>
-      </c>
-      <c r="B11" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="C11" s="16" t="n">
-        <v>151.068714285714</v>
-      </c>
-      <c r="D11" s="16" t="n">
-        <v>38.2295714285714</v>
-      </c>
-      <c r="E11" s="16" t="n">
-        <v>71.8122857142857</v>
-      </c>
-      <c r="F11" s="16" t="n">
-        <v>69.1028571428571</v>
-      </c>
-      <c r="G11" s="14" t="n">
-        <v>9.31528571428572</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>1.57485714285714</v>
-      </c>
-      <c r="I11" s="16" t="n">
-        <v>167.397432996347</v>
-      </c>
-      <c r="J11" s="22" t="n">
-        <v>0.0977</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>18.798</v>
-      </c>
-      <c r="M11" s="16" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="B12" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" s="18" t="n">
-        <v>195.132333333333</v>
-      </c>
-      <c r="D12" s="18" t="n">
-        <v>39.1085</v>
-      </c>
-      <c r="E12" s="18" t="n">
-        <v>80.143</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <v>75.3</v>
-      </c>
-      <c r="G12" s="15" t="n">
-        <v>9.31833333333333</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>1.79916666666667</v>
-      </c>
-      <c r="I12" s="18" t="n">
-        <v>178.524281693897</v>
-      </c>
-      <c r="J12" s="23" t="n">
-        <v>0.1226</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>379</v>
-      </c>
-      <c r="L12" s="15" t="n">
-        <v>20.774</v>
-      </c>
-      <c r="M12" s="18" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>380</v>
-      </c>
-      <c r="B13" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>195.132333333333</v>
-      </c>
-      <c r="D13" s="16" t="n">
-        <v>39.1085</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>80.143</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>75.3</v>
-      </c>
-      <c r="G13" s="14" t="n">
-        <v>9.31833333333333</v>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>1.79916666666667</v>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>178.524281693897</v>
-      </c>
-      <c r="J13" s="22" t="n">
-        <v>0.1226</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="L13" s="14" t="n">
-        <v>20.774</v>
-      </c>
-      <c r="M13" s="16" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>380</v>
-      </c>
-      <c r="B14" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" s="18" t="n">
-        <v>149.9926</v>
-      </c>
-      <c r="D14" s="18" t="n">
-        <v>52.8152</v>
-      </c>
-      <c r="E14" s="18" t="n">
-        <v>77.6606</v>
-      </c>
-      <c r="F14" s="18" t="n">
-        <v>75.8416</v>
-      </c>
-      <c r="G14" s="15" t="n">
-        <v>8.2484</v>
-      </c>
-      <c r="H14" s="9" t="n">
-        <v>1.787</v>
-      </c>
-      <c r="I14" s="18" t="n">
-        <v>162.332346613696</v>
-      </c>
-      <c r="J14" s="23" t="n">
-        <v>0.1651</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>377</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>20.324</v>
-      </c>
-      <c r="M14" s="18" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>380</v>
-      </c>
-      <c r="B15" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="C15" s="16" t="n">
-        <v>221.665090909091</v>
-      </c>
-      <c r="D15" s="16" t="n">
-        <v>37.2651818181818</v>
-      </c>
-      <c r="E15" s="16" t="n">
-        <v>100.463272727273</v>
-      </c>
-      <c r="F15" s="16" t="n">
-        <v>117.458181818182</v>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>7.91209090909091</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>1.68418181818182</v>
-      </c>
-      <c r="I15" s="16" t="n">
-        <v>215.518963920522</v>
-      </c>
-      <c r="J15" s="22" t="n">
-        <v>0.1055</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="L15" s="14" t="n">
-        <v>28.608</v>
-      </c>
-      <c r="M15" s="16" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>380</v>
-      </c>
-      <c r="B16" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="C16" s="18" t="n">
-        <v>190.4386</v>
-      </c>
-      <c r="D16" s="18" t="n">
-        <v>47.0158</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <v>72.7814</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>107.088</v>
-      </c>
-      <c r="G16" s="15" t="n">
-        <v>9.3162</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>1.6808</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>185.890821831519</v>
-      </c>
-      <c r="J16" s="23" t="n">
-        <v>0.0952</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>382</v>
-      </c>
-      <c r="L16" s="15" t="n">
-        <v>20.049</v>
-      </c>
-      <c r="M16" s="18" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
-        <v>380</v>
-      </c>
-      <c r="B17" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="16" t="n">
-        <v>176.534714285714</v>
-      </c>
-      <c r="D17" s="16" t="n">
-        <v>45.582</v>
-      </c>
-      <c r="E17" s="16" t="n">
-        <v>97.1982857142857</v>
-      </c>
-      <c r="F17" s="16" t="n">
-        <v>121.582571428571</v>
-      </c>
-      <c r="G17" s="14" t="n">
-        <v>8.94628571428572</v>
-      </c>
-      <c r="H17" s="6" t="n">
-        <v>1.65685714285714</v>
-      </c>
-      <c r="I17" s="16" t="n">
-        <v>193.035955279126</v>
-      </c>
-      <c r="J17" s="22" t="n">
-        <v>0.0423</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>28.47</v>
-      </c>
-      <c r="M17" s="16" t="n">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -7499,6 +7635,696 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:M17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="B3" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>224.873875</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>51.426875</v>
+      </c>
+      <c r="E3" s="16" t="n">
+        <v>79.514375</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>110.959</v>
+      </c>
+      <c r="G3" s="14" t="n">
+        <v>8.208875</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>0.710875</v>
+      </c>
+      <c r="I3" s="16" t="n">
+        <v>500.540267735832</v>
+      </c>
+      <c r="J3" s="22" t="n">
+        <v>0.0048</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>18.033</v>
+      </c>
+      <c r="M3" s="16" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="B4" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="18" t="n">
+        <v>224.9996</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>59.8344</v>
+      </c>
+      <c r="E4" s="18" t="n">
+        <v>85.172</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>118.3634</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>7.3848</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="I4" s="18" t="n">
+        <v>373.165042543947</v>
+      </c>
+      <c r="J4" s="23" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>23.376</v>
+      </c>
+      <c r="M4" s="18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>225.403142857143</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>50.718</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>74.8847142857143</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>102.72</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>8.483</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.872857142857143</v>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>402.175669000924</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.0117</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>10.993</v>
+      </c>
+      <c r="M5" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>224.914</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>50.29</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>99.938</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>121.1454</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>7.5276</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0.9376</v>
+      </c>
+      <c r="I6" s="18" t="n">
+        <v>400.204833233857</v>
+      </c>
+      <c r="J6" s="23" t="n">
+        <v>0.0128</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="L6" s="15" t="n">
+        <v>28.854</v>
+      </c>
+      <c r="M6" s="18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>223.309</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>42.6395</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>76.9009</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>110.745</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>9.1322</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>1.052</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>325.995300891542</v>
+      </c>
+      <c r="J7" s="22" t="n">
+        <v>0.0172</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>17.351</v>
+      </c>
+      <c r="M7" s="16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>149.9926</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>52.8152</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>77.6606</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>75.8416</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>8.2484</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>1.787</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <v>162.332346613696</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <v>0.1651</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="L8" s="15" t="n">
+        <v>20.324</v>
+      </c>
+      <c r="M8" s="18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>119.5725</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>43.6025</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>52.6261666666667</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>56.389</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>8.07066666666667</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>1.36783333333333</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <v>166.827549144259</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.2719</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>26.594</v>
+      </c>
+      <c r="M9" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>125.2542</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>39.7184</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>59.4492</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>73.224</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>9.3226</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>1.3474</v>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>167.32673415805</v>
+      </c>
+      <c r="J10" s="23" t="n">
+        <v>0.0715</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="L10" s="15" t="n">
+        <v>19.494</v>
+      </c>
+      <c r="M10" s="18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>151.068714285714</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>38.2295714285714</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>71.8122857142857</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>69.1028571428571</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>9.31528571428572</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>1.57485714285714</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <v>167.397432996347</v>
+      </c>
+      <c r="J11" s="22" t="n">
+        <v>0.0977</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>18.798</v>
+      </c>
+      <c r="M11" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>195.132333333333</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>39.1085</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>80.143</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>9.31833333333333</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>1.79916666666667</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>178.524281693897</v>
+      </c>
+      <c r="J12" s="23" t="n">
+        <v>0.1226</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>20.774</v>
+      </c>
+      <c r="M12" s="18" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>195.132333333333</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>39.1085</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>80.143</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>9.31833333333333</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>1.79916666666667</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>178.524281693897</v>
+      </c>
+      <c r="J13" s="22" t="n">
+        <v>0.1226</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="L13" s="14" t="n">
+        <v>20.774</v>
+      </c>
+      <c r="M13" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>149.9926</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>52.8152</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>77.6606</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>75.8416</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>8.2484</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>1.787</v>
+      </c>
+      <c r="I14" s="18" t="n">
+        <v>162.332346613696</v>
+      </c>
+      <c r="J14" s="23" t="n">
+        <v>0.1651</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>20.324</v>
+      </c>
+      <c r="M14" s="18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>221.665090909091</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>37.2651818181818</v>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>100.463272727273</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>117.458181818182</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>7.91209090909091</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>1.68418181818182</v>
+      </c>
+      <c r="I15" s="16" t="n">
+        <v>215.518963920522</v>
+      </c>
+      <c r="J15" s="22" t="n">
+        <v>0.1055</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="L15" s="14" t="n">
+        <v>28.608</v>
+      </c>
+      <c r="M15" s="16" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>190.4386</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>47.0158</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>72.7814</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>107.088</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>9.3162</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>1.6808</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>185.890821831519</v>
+      </c>
+      <c r="J16" s="23" t="n">
+        <v>0.0952</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>20.049</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>176.534714285714</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>45.582</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>97.1982857142857</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>121.582571428571</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>8.94628571428572</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>1.65685714285714</v>
+      </c>
+      <c r="I17" s="16" t="n">
+        <v>193.035955279126</v>
+      </c>
+      <c r="J17" s="22" t="n">
+        <v>0.0423</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>28.47</v>
+      </c>
+      <c r="M17" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -7511,7 +8337,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>402</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7519,13 +8345,13 @@
         <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>386</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7599,7 +8425,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>2</v>
@@ -7607,7 +8433,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>387</v>
+        <v>405</v>
       </c>
       <c r="B10" s="24" t="n">
         <v>233015.6</v>
@@ -7615,7 +8441,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>388</v>
+        <v>406</v>
       </c>
       <c r="B11" s="21" t="n">
         <v>0.085</v>
@@ -7623,7 +8449,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="B12" s="24" t="n">
         <v>0.73</v>
@@ -7631,7 +8457,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>390</v>
+        <v>408</v>
       </c>
       <c r="B13" s="25" t="n">
         <v>154.4</v>
@@ -7639,7 +8465,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>391</v>
+        <v>409</v>
       </c>
       <c r="B14" s="24" t="n">
         <v>130.9</v>
@@ -7647,7 +8473,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>392</v>
+        <v>410</v>
       </c>
       <c r="B15" s="25" t="n">
         <v>170.2</v>
@@ -7655,24 +8481,24 @@
     </row>
     <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>393</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>396</v>
+        <v>414</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>397</v>
+        <v>415</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>398</v>
+        <v>416</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>64</v>
@@ -7680,7 +8506,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>399</v>
+        <v>417</v>
       </c>
       <c r="B19" s="7" t="n">
         <v>594</v>
@@ -7701,7 +8527,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>400</v>
+        <v>418</v>
       </c>
       <c r="B20" s="10" t="n">
         <v>19</v>
@@ -7722,7 +8548,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>401</v>
+        <v>419</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>1</v>
@@ -7768,24 +8594,24 @@
     </row>
     <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>402</v>
+        <v>420</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>396</v>
+        <v>414</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>397</v>
+        <v>415</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>398</v>
+        <v>416</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>64</v>
@@ -7793,7 +8619,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>399</v>
+        <v>417</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>9281.25</v>
@@ -7814,7 +8640,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>400</v>
+        <v>418</v>
       </c>
       <c r="B27" s="10" t="n">
         <v>296.875</v>
@@ -7835,7 +8661,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>401</v>
+        <v>419</v>
       </c>
       <c r="B28" s="7" t="n">
         <v>15.625</v>
@@ -7881,31 +8707,31 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>403</v>
+        <v>421</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>404</v>
+        <v>422</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>405</v>
+        <v>423</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>400</v>
+        <v>418</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>406</v>
+        <v>424</v>
       </c>
       <c r="C34" s="7" t="n">
         <v>1159</v>
@@ -7913,10 +8739,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>399</v>
+        <v>417</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>406</v>
+        <v>424</v>
       </c>
       <c r="C35" s="10" t="n">
         <v>13651</v>
@@ -7924,10 +8750,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>401</v>
+        <v>419</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>406</v>
+        <v>424</v>
       </c>
       <c r="C36" s="7" t="n">
         <v>103</v>
@@ -7935,7 +8761,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>407</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>